<commit_message>
fix(backend): 집계 기준 정립과 입력 검증, 스키마 제약 (v1.5.4.0, SYM-63~72)
- 집계 기준을 화면 목적으로 분리. 대시보드는 활성 TC 만(분모와 분자 함께),
  리포트와 수행 상세는 수행 시점 기록 유지. 두 분기가 헬퍼 하나를 공유한다
- 수행에 편입된 TC 는 기한이 지나도 완전 삭제하지 않는다. 보존하기로 한 기록이
  8일째에 사라져 리포트 총계가 저절로 달라지던 것을 막는다
- 수행에 이미 있는 행은 TC 삭제나 시트 이동 뒤에도 결과를 저장할 수 있다.
  새로 끼어드는 TC 만 막는다
- 검증 추가: 커스텀 필드 타입(생성과 수정 공유), 벌크 삭제 ids, 삭제된 TC 수정,
  임포트의 폴더 시트, 업로드 청크 중단, Alembic 이전 DB 스키마 확인
- 유니크 인덱스 2종 추가(project_members, test_case_sheets). 마이그레이션은
  중복 정리 시 하위 시트를 남는 부모로 옮기고 일반 시트를 폴더보다 우선 보존한다
- TC 목록 엑셀을 leaf_sheet_order 로 정렬해 수행/리포트 엑셀과 기준을 맞춘다

실측: 대시보드 합격률 40.0% -> 30.0%, 교차 프로젝트 집계 누수 pass=504 -> 0
테스트: 백엔드 392 통과(신규 32건)

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VrK5t72J3aeMXh1nFkKgXN
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U176"/>
+  <dimension ref="A1:U198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -14084,6 +14084,1864 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>BUG-113</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>대시보드 전체 모드가 삭제된 TC 의 결과를 분자에 센다</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>- 분모는 활성 TC 로 좁히는데 분자는 결과 행 전체를 센다
+- 실측: TC 를 하나 지우자 합격률이 36.4% 에서 40.0% 로 올랐다
+- 많이 지우면 pass 가 total 을 넘는다</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>- 지운 TC 는 분모와 분자 양쪽에서 빠진다</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>- total 은 11 에서 10 으로 줄었는데 pass 는 4 그대로였다</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>1. TC 를 전부 PASS 로 채운 수행을 만든다
+2. PASS 인 TC 하나를 삭제한다
+3. 대시보드를 연다(수행 선택 없이)</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>실측 API 응답: 삭제 전 total=11 pass=4 rate=36.4, 삭제 후 total=10 pass=4 rate=40.0</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr">
+        <is>
+          <t>SYM-63</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>SEC-016</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>대시보드가 다른 프로젝트 수행의 집계를 돌려준다</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>- run_id 만 보고 그 수행이 이 프로젝트 것인지 확인하지 않는다
+- 권한은 조회 대상 프로젝트만 검사한다</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>- 다른 프로젝트의 수행 번호를 넣으면 0 이 나온다</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>- total=0 인데 pass=504 로 남의 프로젝트 집계가 그대로 나왔다</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>1. 프로젝트 A 의 대시보드를 연다
+2. 쿼리에 프로젝트 B 의 run_id 를 넣는다</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>GET /api/projects/118/dashboard/summary?run_id=27 -&gt; {total:0, pass:504}</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>SYM-64</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>BUG-114</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>지운 TC 의 수행 기록이 7일 뒤 사라져 리포트 총계가 달라진다</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>- 소프트 삭제 TC 를 7일 뒤 완전히 지우면서 결과 행도 같이 사라진다
+- 완료된 수행의 리포트 총계가 시간이 지나면 줄어든다</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>- 수행에 편입된 TC 는 기록 보존을 위해 남긴다</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>- 참조 여부를 보지 않고 기한만으로 지웠다</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>1. 수행에 편입된 TC 를 삭제한다
+2. 8일 뒤 서버를 재시작한다
+3. 그 수행의 리포트를 연다</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>main.py 의 기한 기반 삭제가 TestResult 참조를 보지 않음</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>SYM-65</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>BUG-115</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>커스텀 필드 수정 API 에 타입 검증이 없다</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>- 생성은 허용 목록을 검사하는데 수정은 그대로 저장한다</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>- 생성과 수정이 같은 검증을 쓴다</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>- PUT 으로 임의 문자열이 저장됐다</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>1. 커스텀 필드를 만든다
+2. PUT 으로 field_type 에 허용 목록 밖 값을 보낸다</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>PUT .../custom-fields/1 {field_type:'EVIL_TYPE'} -&gt; 200, DB 에 그대로 저장</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>SYM-66</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>BUG-116</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>시트를 옮긴 TC 가 수행에 남아 결과를 저장할 수 없다</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>- 수행은 한 번 담은 행을 빼지 않는데 결과 제출은 시트 범위를 다시 검사한다
+- 그리드에 보이는데 저장만 400 이라 사라지지도 채워지지도 않는다</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>- 수행에 이미 있는 행은 저장할 수 있다</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>- 400 으로 거부됐다</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>1. 시트 A 만 담은 수행을 만든다
+2. A 의 TC 를 시트 B 로 옮긴다
+3. 수행 상세에서 그 행에 결과를 입력한다</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>testruns.py 의 시트 범위 검사가 기존 결과 행을 예외로 두지 않음</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>SYM-67</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>BUG-117</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>TC 목록 엑셀이 시트 차례를 무시하고 번호로만 정렬한다</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>- 번호는 시트 안 순번이라 시트마다 1부터 시작한다
+- 통합 모드에서 시트가 한 줄씩 번갈아 나온다</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>- 화면의 시트 차례를 따른다(수행·리포트 엑셀과 같은 기준)</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>- 가-1, 나-1, 다-1, 가-2 순으로 섞였다</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>1. 시트 여러 개에 TC 를 넣는다
+2. TC 관리에서 엑셀 내보내기(통합 모드)</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>export_testcases 가 order_by(TestCase.no) 만 사용</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr">
+        <is>
+          <t>SYM-68</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>BUG-118</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>임포트가 폴더 시트에 TC 를 넣고 벌크 삭제가 500 을 낸다</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>- 임포트 네 경로가 폴더 여부를 보지 않는다. 폴더에 들어간 TC 는 수행에 담을 수 없다
+- 벌크 삭제의 ids 에 숫자가 아닌 값이 오면 500 이 난다</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>- 폴더 임포트는 400, 잘못된 ids 도 400</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>- 임포트는 201 로 통과, ids=abc 는 500</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>1. 폴더 시트를 만든다
+2. 같은 이름의 시트가 든 엑셀을 임포트한다
+3. DELETE .../testcases/bulk?ids=abc 를 호출한다</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>폴더에 TC 임포트 201, ids=abc 에서 Internal server error</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>SYM-69</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>BUG-119</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>멤버와 시트 이름 중복을 DB 가 막지 않는다</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>- 조회 후 삽입만 해서 동시 요청을 막지 못한다
+- 멤버가 둘이면 권한 판정이 비결정적이고, 시트가 둘이면 rename/delete 가 한쪽만 건드린다</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>- DB 제약으로 막는다</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>- 애플리케이션 검사만 있었다</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>1. 같은 멤버 추가 요청을 동시에 두 번 보낸다</t>
+        </is>
+      </c>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>models.py 의 인덱스가 unique 가 아님</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>SYM-70</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>SEC-017</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>업로드 크기 제한이 버퍼를 다 채운 뒤에야 걸리고 삭제된 TC 를 수정할 수 있다</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>- read() 로 전부 읽은 뒤 길이를 재서, 제한을 넘는 파일도 버퍼에 통째로 올라온 뒤 거절한다
+- 삭제된 TC 를 수정 API 로 계속 고칠 수 있다</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>- 제한을 넘는 순간 끊고, 지운 TC 는 404</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>- 전량 적재 후 413, 삭제된 TC 수정은 200</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>1. 제한을 넘는 파일을 업로드한다
+2. 삭제한 TC 에 PUT 을 보낸다</t>
+        </is>
+      </c>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>attachments.py 와 import_service.py 의 크기 검사 위치</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr">
+        <is>
+          <t>SYM-71</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>BUG-120</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Alembic 이전 DB 를 검증 없이 최신으로 표시한다</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>- 테이블은 있고 alembic_version 만 없으면 스키마를 보지 않고 head 로 표시한다
+- 그 사이 마이그레이션이 전부 건너뛰어진다</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>- 표지 컬럼을 확인하고, 최신이 아니면 멈추고 알린다</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>- 구버전 스키마가 최신으로 표시됐다</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>1. alembic_version 이 없는 구버전 DB 로 서버를 띄운다</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>main.py 의 stamp(head) 경로에 스키마 검사 없음</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr">
+        <is>
+          <t>SYM-72</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>BUG-121</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>수행 그리드에서 0.3초 안에 다른 행을 편집하면 앞 행 저장이 취소된다</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>- 저장 디바운스 타이머가 행별이 아니라 전역 하나다
+- 에러도 토스트도 없이 입력이 사라진다</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>- 행마다 따로 저장된다</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>- 뒤에 편집한 행만 저장됐다</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>1. 수행 상세에서 A 행 결과를 입력한다
+2. 0.3초 안에 B 행을 입력한다
+3. 새로고침한다</t>
+        </is>
+      </c>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>TestRunManager 는 전역 타이머, TestCaseGrid 는 행별 키로 비대칭</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr">
+        <is>
+          <t>SYM-73</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>BUG-122</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>타이머가 잰 소요 시간이 저장되지 않는다</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>- 경과 시간을 화면에만 찍고 저장 경로에 넣지 않는다
+- 매뉴얼은 결과 입력 시 기록된다고 안내하고 수행 엑셀에도 칸이 있다</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>- 잰 시간이 결과와 함께 저장된다</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>- 실 DB 결과 5,209건 중 기록된 것이 0건이었다</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>1. 수행 상세에서 타이머를 켠다
+2. A 행에서 B 행으로 옮긴다
+3. 수행을 다시 연다</t>
+        </is>
+      </c>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>test_results 의 duration_sec NOT NULL 집계 0건</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr">
+        <is>
+          <t>SYM-74</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>BUG-123</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>프로젝트 설명을 지우면 저장되지 않는데 성공 메시지가 뜬다</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>- 빈 문자열을 undefined 로 바꿔 보내서 키가 통째로 빠진다
+- 백엔드는 보내지 않은 필드를 건드리지 않는다</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>- 지운 설명이 저장된다</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>- 성공 토스트가 뜨지만 값은 그대로 남고, 다시 들어가면 되살아난다</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>1. 프로젝트 설정에서 설명을 전부 지운다
+2. 저장한다
+3. 다른 탭에 갔다가 돌아온다</t>
+        </is>
+      </c>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>PUT 에 description 키를 빼고 보내면 기존 값이 유지됨(실측)</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr">
+        <is>
+          <t>SYM-75</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>SEC-018</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>아이디에 든 HTML 이 관리자 화면에서 실행된다</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>- 사용자명을 dangerouslySetInnerHTML 에 끼워 넣는다
+- i18n 이 값을 이스케이프하지 않는 설정이고 아이디에 문자 제한이 없다</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>- 아이디는 글자로만 보인다</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>- img 태그가 DOM 에 삽입됐다</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>1. HTML 이 든 아이디로 가입한다
+2. 관리자가 그 계정 비밀번호를 초기화한다
+3. 완료 모달이 뜬다</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>테스트에서 container.querySelector('img') 가 실제 요소를 반환</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R190" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T190" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U190" t="inlineStr">
+        <is>
+          <t>SYM-76</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>BUG-124</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>영어로 쓰면 새 행의 우선순위가 번역문으로 저장된다</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>- 새 행 기본값에 화면 표기용 번역 문자열을 넣는다
+- DB 값은 한글 5종인데 영어에서는 Normal 이 저장된다</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>- 로케일과 무관하게 DB 값이 저장된다</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>- priority 에 Normal 이 들어가 색상과 선택지에서 빠지고 통계가 갈린다</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>1. 언어를 영어로 바꾼다
+2. TC 관리에서 행을 추가한다</t>
+        </is>
+      </c>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>TestCaseGrid 의 새 행 기본값이 t('priority.normal')</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>SYM-77</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>BUG-125</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>찾기 바꾸기가 필터로 숨은 행까지 바꾸고 수행 그리드 메모의 줄바꿈이 사라진다</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>- 바꾸기가 필터와 무관하게 로드된 모든 행을 돈다
+- 수행 그리드 Remarks 에 큰 편집기를 안 달아 기본 입력칸이 열리고 줄바꿈이 지워진다</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>- 보이는 행만 바꾸고, 여러 줄 메모는 줄바꿈을 지킨다</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>- 화면에 없는 행까지 바뀌고 건수도 그것을 포함했다</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>1. 컬럼 필터를 걸어 행을 좁힌다
+2. 검색어를 넣고 모두 바꾸기를 누른다
+3. 수행 그리드에서 여러 줄 메모를 열었다 닫는다</t>
+        </is>
+      </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>forEachNode 사용, Remarks 컬럼에 cellEditor 미지정</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>SYM-78</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>BUG-126</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>관리자 매뉴얼 안내 박스가 다크모드에서 읽히지 않는다</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>- 배경색만 고정값으로 두고 글자색을 지정하지 않았다
+- 다크모드에서 밝은 배경에 밝은 글자가 된다</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>- 두 테마 모두 읽힌다</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>- 대비 1.14 대 1 로 글자가 보이지 않았다</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>1. 다크모드로 바꾼다
+2. 운영 매뉴얼의 데이터베이스 절을 연다</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>사용자 매뉴얼의 같은 스타일은 v1.5.1.1 에서 이미 토큰으로 고쳐졌음</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>SYM-79</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>BUG-127</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>커스텀 필드 컬럼의 Ctrl+D 와 되돌리기가 값을 바꾸지 않는데 완료 메시지가 뜬다</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>- 값을 최상위 속성에 쓰는데 컬럼은 custom_fields 를 읽는다
+- 저장 페이로드의 키도 백엔드 스키마에 없어 버려진다</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>- 채운 값이 화면과 DB 에 반영된다</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>- 셀은 그대로인데 N개 채움 토스트가 떴다</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>1. 커스텀 필드를 만든다
+2. 그 컬럼의 셀 하나를 채운다
+3. 여러 행을 선택하고 Ctrl+D 를 누른다</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>Ctrl+D 와 undo 가 node.data[field] 에 직접 대입</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>SYM-80</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>BUG-128</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>비교 화면에서 늦게 온 응답이 최신 결과를 덮는다</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>- 수행 선택기는 로딩 중에도 떠 있어 응답 전에 다른 수행을 고를 수 있다
+- 세대 번호가 없어 먼저 보낸 요청이 나중에 도착하면 화면을 덮는다</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>- 지금 고른 수행의 결과만 보인다</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>- 새 수행이 선택된 채 옛 결과가 표시됐다</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>1. 비교 화면에서 기준 수행을 고른다
+2. 응답 전에 다른 수행으로 바꾼다</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>간헐</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>CompareView.loadResults 에 세대 번호 없음</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>SYM-81</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>BUG-129</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>대시보드 담당자별 표가 늘 비어 있고 일괄 삭제는 전부 실패해도 성공 메시지를 띄운다</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>- 담당자 필드는 v1.2.0 에서 없어졌고 API 는 빈 배열만 돌려주는데 화면은 표를 그린다
+- 프로젝트 일괄 삭제가 개별 실패를 로그로만 남기고 늘 성공 토스트를 띄운다</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>- 쓰지 않는 표는 그리지 않고, 실패는 실패로 알린다</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>- 빈 표가 계속 보이고, 하나도 못 지웠는데 지워진 줄 안다</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>1. 대시보드를 연다
+2. 프로젝트를 여러 개 선택해 삭제하고 서버가 거절하게 한다</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>assignee_summary 가 return [] 스텁</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>SYM-82</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>BUG-130</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>i18n 키 누락과 미선언 CSS 토큰, 필터 아이콘 대비</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>- 정의되지 않은 키 두 곳이 화면에 키 문자열로 노출된다
+- 선언되지 않은 토큰 세 곳이 폴백 고정색으로 그려져 다크모드 대비가 떨어진다
+- 필터가 걸린 컬럼 아이콘이 안 걸린 것보다 흐리다</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>- 키와 토큰이 실제로 선언돼 있고, 필터가 걸린 컬럼이 눈에 띈다</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>- saveFailed 와 deleteField 가 그대로 노출, 아이콘 대비 1.03 대 1</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>1. 프로젝트 설정에서 이름 저장을 실패시킨다
+2. 컬럼 필터를 건 뒤 헤더 아이콘을 본다</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>i18n 키 대조 2건 누락, var(--danger) 3곳 미선언</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>SYM-83</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>BUG-131</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>trivial</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>버전 표기가 실제 릴리즈와 어긋나고 언어를 바꿔도 수행 그리드 헤더가 그대로다</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>- 백엔드 앱 버전과 package.json 이 일곱 번의 릴리즈 동안 1.4.0.1 에 멈춰 있었다
+- 화면 푸터는 1.5.2.0 이었다
+- 수행 그리드 컬럼 정의가 번역 함수를 의존성에 넣지 않아 언어 전환이 반영되지 않는다</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>- 네 곳의 버전이 릴리즈 노트와 같고, 언어 전환이 헤더에 반영된다</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>- 세 곳이 어긋났고 헤더는 옛 언어로 남았다</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>1. /docs 에서 API 버전을 본다
+2. 언어를 영어로 바꾸고 수행 그리드 헤더를 본다</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>릴리즈 v1.5.3.0 대비 main.py 1.4.0.1, package.json 1.4.0.1, 푸터 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>BE 1.5.3.0 / FE 1.5.2.0</t>
+        </is>
+      </c>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>SYM-84</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(release): v1.5.5.1 릴리즈 노트와 버전 표기 (SYM-85)
빌드 수정 커밋에서 빠뜨린 릴리즈 노트 절과 버전 사본을 채운다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VrK5t72J3aeMXh1nFkKgXN
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U198"/>
+  <dimension ref="A1:U199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -15942,6 +15942,89 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>BUG-132</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>프로덕션 빌드가 타입 오류로 실패한다</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>- npm run build 의 tsc -b 단계가 타입 오류로 죽는다
+- CI 의 Frontend 잡이 실패한다</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>- 빌드가 통과한다</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>- node API 를 쓰는 검사 테스트에서 모듈을 못 찾고, 지운 API 를 모킹하던 테스트가 남아 있었다</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>1. frontend 에서 npm run build 를 실행한다</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>error TS2307 Cannot find module 'node:fs', error TS2339 Property 'assignee' does not exist</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>FE 1.5.3.0</t>
+        </is>
+      </c>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>SYM-85</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: 응답 계약과 로케일, 남은 검증 공백 (v1.5.6.0, SYM-86~94)
- 리포트 요약·PDF·엑셀에 executed(pass+fail+block) 표기. pass_rate 만 분모가
  수행분이고 나머지 넷은 전체라, 이름만으로 알 수 없던 분모를 드러낸다.
  계산은 _summary_sql 한 곳에서 한다
- 쓰이지 않던 대시보드 응답 스키마 5종 제거. response_model 로 붙이는 순간
  pass_ 키로 나가 화면이 조용히 비는 모양이었다
- 가입 직후 관리자 판정을 다시 해 동시 가입 경쟁을 막는다(SQLite 전제를 주석에 명시)
- TC ID 1~50자 검증을 생성과 수정에 건다. 응답 스키마에는 걸지 않는다.
  기존 값이 규칙을 어길 때 조회까지 막히면 고칠 방법이 없다
- 시트 이름 변경의 번호 충돌을 이유 있는 400 으로 바꾼다. 미리 "그 이름을 쓰는
  TC 가 있으면 거절" 로 막으면 부딪히지 않는 경우까지 막는다
- 시트 이동은 보내지 않은 필드를 건드리지 않는다
- 내보내기 모달 7문구와 사전조건 안내 3문구를 i18n 으로, 날짜 프리셋을 로컬 기준으로
- 리포트 전용 응답 타입 정의. 엔티티를 그대로 쓰면 오지 않는 필드까지 선언하게 된다

검증에서 되돌린 것: 완료 전 동기화는 완료 순간에 새 TC 를 NS 로 끌어들여 총계와
비율을 바꾸므로 뺐다. rename 의 사전 차단도 부딪히지 않는 경우를 막아 제약 판정에 맡겼다.

테스트: 백엔드 404, 프론트 482 통과. 빌드와 린트 오류 0

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VrK5t72J3aeMXh1nFkKgXN
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U199"/>
+  <dimension ref="A1:U208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16025,6 +16025,759 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>BUG-133</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>리포트 비율의 분모가 서로 달라 합이 100 이 되지 않는다</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>- pass_rate 만 분모가 수행분(pass+fail+block)이고 나머지 넷은 전체다
+- 이름만으로는 어느 쪽인지 알 수 없다</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>- 소비자가 분모를 알 수 있다</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>- 다섯을 더하면 100 이 되리라 기대하게 된다</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>1. 미수행이 섞인 수행의 리포트를 조회한다
+2. 다섯 비율을 더한다</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>TC 4건 중 2 PASS / 1 FAIL / 1 미수행이면 pass_rate 66.7, fail_rate 25.0</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>SYM-86</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>BUG-134</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>쓰이지 않는 대시보드 응답 스키마가 붙는 순간 화면을 비운다</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>- 대시보드 스키마 5개가 pass_ 로 선언하고 파이썬 model_dump 오버라이드로 이름을 바꾼다
+- 아무 데서도 쓰지 않지만 response_model 로 붙이면 FastAPI 직렬화가 그 오버라이드를 건너뛴다</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>- 나중에 손대도 터지지 않는다</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>- 응답 키가 pass_ 가 되어 카드와 도넛이 조용히 빈다</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>1. 대시보드 라우트에 response_model=DashboardSummary 를 붙인다
+2. 대시보드를 연다</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>schemas.py 의 5개 모델이 라우트에서 import 되지 않음</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>SYM-87</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>SEC-019</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>최초 관리자 승격에 동시 가입 경쟁이 있다</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>- User.count()==0 을 보고 관리자를 준다
+- 같은 순간에 두 가입이 들어오면 둘 다 0 을 보고 둘 다 관리자가 된다</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>- 최초 관리자는 한 명이다</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>- 조회와 삽입 사이가 열려 있었다</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>1. 빈 DB 에 가입 요청 두 건을 동시에 보낸다</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>미확인</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>routes/auth.py 의 register 가 삽입 전 count 만 본다</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>SYM-88</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>BUG-135</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>TC ID 에 길이 검증이 없어 컬럼 제한을 넘는 값이 저장된다</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>- 컬럼은 String(50) 인데 SQLite 는 길이를 강제하지 않는다
+- 빈 문자열도 통과한다</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>- 1자 이상 50자 이하만 받는다</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>- 60자 TC ID 와 빈 값이 그대로 저장됐다</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>1. tc_id 에 60자 문자열을 넣어 TC 를 만든다</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>schemas.py 의 tc_id 에 min_length/max_length 없음</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>SYM-89</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>BUG-136</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>TC 만 남은 이름으로 시트를 바꾸면 이유를 알 수 없는 오류가 난다</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>- 시트를 지워도 TC 의 sheet_name 은 남는다
+- rename 중복 검사가 시트 테이블만 봐서 통과한 뒤 유니크 제약에 걸린다</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>- 400 으로 이유를 알려 준다</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>- 데이터 제약 조건에 걸렸습니다 라는 409 만 나온다</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>1. 시트에 TC 를 넣고 시트만 지운다
+2. 다른 시트를 그 이름으로 바꾼다</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>sheets.py 의 rename 중복 검사가 TestCase.sheet_name 을 보지 않음</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>SYM-90</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>BUG-137</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>시트 이동이 보내지 않은 필드를 바꾼다</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>- reopen 은 동기화를 부르는데 complete 는 부르지 않는다
+- move 의 parent_id 가 Optional 기본 None 이라 안 보낸 요청도 시트를 루트로 끌어낸다</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>- 완료 전에 한 번 맞추고, 보내지 않은 필드는 건드리지 않는다</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>- 상세를 열지 않고 완료하면 그 TC 가 영영 안 들어오고, sort_order 만 보낸 요청이 부모를 지운다</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>1. 진행 중 수행이 있는 프로젝트에 TC 를 더한다
+2. 상세를 열지 않고 완료한다</t>
+        </is>
+      </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>testruns.py 의 complete 에 sync_run_results 없음, sheets.py 의 move 가 조건 없이 대입</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>SYM-91</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>BUG-138</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>영어 화면에 한글 문구가 그대로 나온다</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>- 내보내기 옵션 모달 일곱 문구가 하드코딩이다
+- 사전조건 참조 안내 세 문구도 한글 고정이다</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>- 로케일을 따른다</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>- 영어로 바꿔도 한글이 섞여 나온다</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>1. 언어를 영어로 바꾼다
+2. TC 관리에서 Excel Export 를 연다</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>TestCaseGrid 의 모달 문구와 utils/precondition.ts 의 반환 문자열</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>SYM-92</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>BUG-139</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>대시보드 날짜 프리셋이 UTC 기준이라 경계일이 밀린다</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>- toISOString 을 써서 UTC 날짜를 낸다
+- KST 에서 자정부터 오전 9시 사이에 하루 전 날짜가 된다</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>- 브라우저 로컬 날짜를 쓴다</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>- 새벽에 7일 프리셋을 누르면 8일 전부터 잡힌다</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>1. KST 새벽에 대시보드를 연다
+2. 7일 프리셋을 누른다</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>Dashboard.tsx 의 new Date(...).toISOString().split('T')[0]</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>SYM-93</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>BUG-140</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>리포트 응답 타입이 실제와 달라 컴파일러가 보호하지 못한다</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>- top_failures 를 TestResult[] 로 선언하지만 실제로는 네 필드짜리 조각이 온다
+- project 와 test_run 도 엔티티 전체가 아니다</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>- 실제 응답 모양을 선언한다</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>- 필수로 선언한 필드가 항상 undefined 이고 방어 코드만 화면을 지탱했다</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>1. ReportData 타입과 reports.py 의 응답 조립부를 대조한다</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr">
+        <is>
+          <t>항상</t>
+        </is>
+      </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>is_private, project_id, created_by 등이 응답에 없음</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 / FE 1.5.3.1</t>
+        </is>
+      </c>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>SYM-94</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(deps): 프론트·백엔드 의존성 취약점 8건 해소 (v1.5.7.0, SYM-95 SYM-96)
프론트: axios 의 NO_PROXY 우회 SSRF 와 validateStatus 프로토타입 오염,
react-router 의 turbo-stream 역직렬화 RCE, form-data CRLF 주입을 닫는다.
axios, react-router-dom, dompurify 를 올리면 하위 form-data 와
follow-redirects 도 함께 올라간다.

백엔드: requirements.txt 에서 python-multipart 만 버전 핀이 없어 0.0.22 가
설치돼 있었다. 헤더 무제한 처리 DoS 와 세미콜론 쿼리스트링 2차 파싱 DoS 에
해당한다. ==0.0.32 로 핀하고 사유를 주석으로 남긴다.

프론트 npm audit --omit=dev: high 4 / moderate 2 -> 0건
백엔드 python-multipart OSV: 12건 -> 0건
검증: 프론트 빌드 + vitest 482건, 백엔드 테스트 184건 통과

routes/attachments.py 의 UploadFile 경로가 이 파서를 직접 탄다.
배포 환경은 pip install -r requirements.txt 재실행이 필요하다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U208"/>
+  <dimension ref="A1:U210"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16778,6 +16778,230 @@
         </is>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>BUG-141</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>프론트 의존성에 axios SSRF, react-router RCE 등 취약점 6건</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>- npm audit --omit=dev 에서 high 4건, moderate 2건이 잡힌다.
+- axios 1.13.6: NO_PROXY 호스트명 정규화 우회로 인한 SSRF, validateStatus 병합 경로의 프로토타입 오염 인증 우회.
+- react-router 7.13.1: 벤더링된 turbo-stream v2 의 TYPE_ERROR 역직렬화로 임의 생성자 호출(미인증 RCE).
+- form-data 4.0.5: 멀티파트 필드명/파일명 미이스케이프로 인한 CRLF 주입.
+- dompurify 3.3.3, follow-redirects 는 moderate.</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>- 프로덕션 의존성에 알려진 high 취약점이 없어야 한다.</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>- high 4 / moderate 2, 합계 6건.</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>1. tc_manager/frontend 에서 npm audit --omit=dev 실행
+2. axios, react-router, form-data, dompurify 항목 확인</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>- npm audit --omit=dev 출력. axios 취약 범위 1.0.0 - 1.17.0, react-router 6.0.0 - 7.18.1.</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰. 전체 프로젝트 보안 점검 중 확인.</t>
+        </is>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>원인: - 세 패키지 모두 캐럿 범위로 두었으나 lockfile 이 갱신되지 않아 취약 버전에 머물렀다.
+수정 내용: - axios, react-router-dom, dompurify 를 최신으로 올렸다. 하위 form-data, follow-redirects 도 함께 갱신됐다.
+- tsc -b &amp;&amp; vite build 통과, vitest 482건 통과 확인
+- npm audit --omit=dev 결과 0건</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>- 이 레포는 CI(.github/workflows/ci.yml)가 있으므로 audit 게이트를 붙일 자리가 있다. 별도 이슈로 다룬다.</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>- 프론트 전반. axios 는 모든 API 호출 경로, react-router 는 라우팅 전체, dompurify 는 MarkdownCell/PreconditionCell 의 XSS 방어.</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>v1.5.6.0</t>
+        </is>
+      </c>
+      <c r="S209" t="inlineStr">
+        <is>
+          <t>- v1.5.7.0</t>
+        </is>
+      </c>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>SYM-95</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>BUG-142</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>python-multipart 에 버전 핀이 없어 헤더 무제한 DoS 버전이 설치된다</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>- requirements.txt 의 python-multipart 에만 버전 핀이 없어 0.0.22 가 설치돼 있었다.
+- 0.0.22 는 멀티파트 파트 헤더 무제한 처리 DoS(GHSA-pp6c-gr5w-3c5g, high)와 세미콜론 쿼리스트링 2차 파싱 DoS(GHSA-5rvq-cxj2-64vf, high)에 해당한다.
+- 그 외 moderate 1건, low 3건을 포함해 12건이 잡힌다.</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>- 파일 업로드를 받는 의존성에 알려진 high 취약점이 없어야 한다.</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>- OSV 조회 결과 python-multipart 0.0.22 에 취약점 12건.</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>- routes/attachments.py 가 UploadFile 로 첨부를 받으므로 이 파서가 요청 경로에 직접 놓인다.</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>1. requirements.txt 에서 python-multipart 행에 버전 지정이 없음을 확인
+2. pip show python-multipart 로 설치 버전이 0.0.22 임을 확인
+3. OSV API 에 PyPI/python-multipart/0.0.22 로 조회</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>- OSV API 응답 12건. GHSA-pp6c-gr5w-3c5g 는 0.0.27 에서, GHSA-5rvq-cxj2-64vf 는 0.0.30 에서 수정.</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰. 전체 프로젝트 보안 점검 중 확인.</t>
+        </is>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>원인: - requirements.txt 의 다른 패키지는 전부 == 로 고정했는데 python-multipart 만 핀 없이 두어, 설치 시점에 따라 임의 버전이 들어왔다.
+수정 내용: - requirements.txt 에 python-multipart==0.0.32 로 핀하고 사유를 주석으로 남겼다.
+- 설치 후 OSV 재조회 0건 확인
+- test_security.py, test_attachment_bulk.py, test_input_validation.py 184건 통과</t>
+        </is>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>- 버전 핀 자체가 가드다. requirements-dev.txt 가 -r requirements.txt 를 참조하므로 CI 전 경로에 전파된다.</t>
+        </is>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>- POST /api/attachments 등 멀티파트를 받는 전 엔드포인트. 인증은 있으나 로그인 사용자가 DoS 를 유발할 수 있었다.</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>v1.5.6.0</t>
+        </is>
+      </c>
+      <c r="S210" t="inlineStr">
+        <is>
+          <t>- v1.5.7.0</t>
+        </is>
+      </c>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>SYM-96</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 토큰 폐기 수단, 접근성 검사, E2E 고정 대기 제거 (v1.6.0.0, SYM-100~103)
users.token_version 을 두고 토큰의 ver 와 요청마다 대조한다. 비밀번호 변경,
관리자 초기화, 계정 복구, 로그아웃 네 경로에서 값을 올려 옛 토큰을 끊는다.
로그인 유지는 3650일에서 30일로 줄였다.

axe-core 검사를 컴포넌트 10건과 화면 5건으로 넣고 CI e2e 에 붙였다. 검사가
잡은 것은 색 대비 7건, 이름 없는 요소 5건, 라벨 미연결 2건, 모달 역할 1건이다.
검색 드롭다운을 Escape 로 닫는 동작도 함께 넣었다.

회귀 E2E 6개 스펙의 waitForTimeout 82건을 응답 대기와 상태 단언으로 바꿨다.
그 과정에서 단언이 없거나 조건부로 건너뛰던 테스트 12건이 드러나 검증을 넣었다.
권한 검사 2건은 소스 문자열 검사에서 HTTP 호출로 바꿨다.

CI 의 타입 검사가 루트 tsconfig(files: [])를 보느라 검사 대상이 0 개였다.
tsc -b 로 바꿨다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U210"/>
+  <dimension ref="A1:U214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -17002,6 +17002,350 @@
         </is>
       </c>
     </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>SEC-020</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>로그인 유지 토큰이 10년이고 폐기할 수단이 없다</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>- 로그인 화면에서 로그인 유지를 켜면 발급되는 JWT 의 만료가 3650일이다.
+- 서버에 토큰을 무효화할 수단이 없다. jti, 블랙리스트, 토큰 버전 중 어느 것도 없다.
+- 로그아웃은 쿠키만 지운다. 같은 토큰을 Authorization 헤더에 실으면 계속 통한다.</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>- 로그인 유지 기간이 상식적인 범위여야 한다.
+- 비밀번호를 바꾸면 그 전에 발급된 토큰이 전부 막혀야 한다.
+- 유출을 알아챈 뒤 대응할 수단이 있어야 한다.</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>- 한 번 유출된 토큰으로 10년간 계정을 쓸 수 있다.
+- 비밀번호를 바꿔도 기존 토큰은 그대로 유효하다.</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>1. 로그인 유지를 켜고 로그인한다.
+2. 응답 본문의 access_token 값을 저장한다.
+3. 로그아웃한다.
+4. 저장한 토큰을 Authorization: Bearer 헤더에 실어 GET /api/auth/me 를 호출한다.
+5. 비밀번호를 변경한 뒤 4번을 다시 호출한다.</t>
+        </is>
+      </c>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>- backend/routes/auth.py:145 timedelta(days=3650)
+- backend/auth.py 전체에 jti/blacklist/token_version 정의 없음
+- backend/routes/auth.py:179 로그아웃이 delete_cookie 만 수행</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰 (프로젝트 수준 평가 중 Codex 교차 검증에서 발견)</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>BE 1.5.5.0</t>
+        </is>
+      </c>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>SYM-100</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>ENH-049</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>접근성 속성이 없어 스크린리더로 쓸 수 없다</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>- tsx 88 개 파일에서 aria 속성과 role 사용이 4 회다.
+- 아이콘만 있는 버튼(다크모드 토글, 시트 닫기 등)에 이름이 없다.
+- 모달에 dialog 역할과 제목 연결이 없다.
+- 접근성을 검사하는 자동 테스트가 없다.</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>- 주요 화면 네 곳에서 axe-core 심각도 serious 이상 위반이 0 건이다.
+- 아이콘 버튼과 폼 입력에 접근 가능한 이름이 붙는다.
+- CI 가 위반을 막는다.</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>- [ ] axe-core 기반 E2E 검사가 로그인·프로젝트 목록·TC 관리·대시보드를 검사한다
+- [ ] serious 이상 위반 0 건
+- [ ] CI e2e 잡에서 함께 돌아간다
+- [ ] 검사가 실제로 위반을 잡는지 일부러 깨뜨려 확인한다</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>- QA 도구가 접근성을 못 갖추면 제품 성격과 어긋난다.
+- 공개 레포라 외부에서 먼저 지적당할 자리다.
+- 지금 넣지 않으면 화면이 늘수록 소급 비용이 커진다.</t>
+        </is>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>- WCAG AAA 대응
+- 키보드 내비게이션 전면 재설계
+- ag-grid 내부가 만드는 DOM 의 위반</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>FE 1.5.4.0</t>
+        </is>
+      </c>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>SYM-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>ENH-050</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>E2E 가 고정 대기에 의존해 불안정하다</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>- 회귀 스펙에서 waitForTimeout 호출이 148 회다. 캡처 전용 스펙을 빼도 82 회다.
+- 같은 자리에서 명시적 expect 대기는 115 회다.
+- 느린 러너에서는 먼저 깨지고 빠른 러너에서는 불필요하게 기다린다.</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>- 회귀 스펙의 고정 대기가 web-first 단언으로 바뀐다.
+- 대기 시간이 줄고 결과가 환경에 덜 흔들린다.</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>- [ ] regression-full, tc-management, v060-features, project, admin, auth 스펙의 waitForTimeout 제거
+- [ ] E2E 가 그대로 통과한다
+- [ ] 캡처 전용 스펙은 그대로 둔다</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>- CI e2e 잡이 8 분대이고 그 상당 부분이 고정 대기다.
+- QA 엔지니어의 공개 레포에서 가장 먼저 지적받는 안티패턴이다.</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>- 캡처 전용 스펙(capture-*.spec.ts)의 고정 대기
+- E2E 스펙 구조 재설계</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>FE 1.5.4.0</t>
+        </is>
+      </c>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>SYM-102</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>BUG-143</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>CI 의 타입 검사가 아무 파일도 보지 않는다</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>- CI frontend 잡의 타입 검사 단계가 npx tsc --noEmit 이다.
+- 루트 tsconfig.json 은 files 가 빈 배열이고 참조만 들고 있어, 이 명령은 검사 대상이 0 개다.
+- 타입 오류가 있어도 이 단계는 항상 통과한다.</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>- 컴파일되지 않는 코드가 있으면 타입 검사 단계에서 멈춰야 한다.</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>- 타입 검사는 통과하고, 뒤의 빌드 단계(tsc -b)에서야 깨진다.
+- v1.5.5.1 의 '프로덕션 빌드가 깨지던 타입 오류' 가 이 구멍으로 새어나간 건이다.</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>1. frontend/src 의 아무 컴포넌트에 없는 prop 을 넘기는 코드를 넣는다.
+2. cd frontend &amp;&amp; npx tsc --noEmit 을 돌린다. 종료코드 0 이다.
+3. npx tsc -b --force 를 돌린다. TS2322 가 난다.</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>- frontend/tsconfig.json: {"files": [], "references": [...]}
+- 실측: 같은 코드에서 tsc --noEmit 은 EXIT=0, tsc -b 는 TS2322</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰 (접근성 작업 중 QA 교차 검증에서 발견)</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>FE 1.5.5.0</t>
+        </is>
+      </c>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>SYM-103</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(log): 이슈 로그 종결 칸 동기화 (SYM-100~103)
issuelog sync 가 트래커에서 원인·수정 내용·재발 방지·영향 범위를 가져와
빈 칸 12개를 채우고 상태 4건을 완료로 맞췄다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -17079,14 +17079,45 @@
           <t>- 코드 리뷰 (프로젝트 수준 평가 중 Codex 교차 검증에서 발견)</t>
         </is>
       </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>원인: * `backend/routes/auth.py:145` 가 로그인 유지에 `timedelta(days=3650)` 을 줬다.
+* JWT 는 발급하면 만료까지 서버가 손댈 수 없는데 폐기 경로를 두지 않았다. `jti`, 블랙리스트, 토큰 버전 중 어느 것도 없었다.
+* 로그아웃은 쿠키만 지웠고, `_extract_token` 이 Authorization 헤더도 받으므로 같은 토큰이 그대로 통했다.
+수정 내용: * `users.token_version` 추가(마이그레이션 `c2f8a90b3d14`). 토큰에 `ver` 를 실어 `get_current_user` 에서 요청마다 대조한다.
+* 비밀번호 변경, 관리자 초기화, 계정 복구, 로그아웃 네 경로에서 버전을 올린다.
+* 로그인 유지 만료를 30일로 줄였다(`REMEMBER_ME_DAYS`).
+* DB 값을 `or 0` 으로 정규화한다. NULL 이면 `ver` 없는 토큰이 통과하는 쪽으로 열린다.
+* `services/schema_guard.py` 표지에 `token_version` 을 넣었다. 없는 DB 를 head 로 표시하면 인증이 통째로 죽는다.</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>* `backend/test_token_revocation.py` 8건. 비밀번호 변경·관리자 초기화·로그아웃 뒤 옛 토큰이 401 인지, 남의 비밀번호 변경이 내 토큰을 건드리지 않는지, 로그인 유지가 31일을 넘지 않는지, `ver` 없는 토큰이 막히는지 검사한다.
+* `backend/test_account_requests.py` 에 복구 경로용 1건 추가.
+* `tests_unit/test_schema_guard.py` 에 `token_version` 누락 검사 1건 추가.</t>
+        </is>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>* 배포 후 모든 사용자가 한 번 다시 로그인해야 한다. 기존 토큰에는 `ver` 가 없어 전부 거부된다.
+* 로그아웃하면 그 계정의 다른 기기 세션도 함께 끊긴다.
+* `alembic_version` 이 없는 구형 DB 는 기동을 멈춘다.</t>
+        </is>
+      </c>
       <c r="R211" t="inlineStr">
         <is>
           <t>BE 1.5.5.0</t>
         </is>
       </c>
+      <c r="S211" t="inlineStr">
+        <is>
+          <t>* BE 1.6.0.0 (커밋: a8d2063)</t>
+        </is>
+      </c>
       <c r="T211" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U211" t="inlineStr">
@@ -17156,6 +17187,24 @@
 - 지금 넣지 않으면 화면이 늘수록 소급 비용이 커진다.</t>
         </is>
       </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>검사를 두 층으로 넣었다. `src/test/accessibility.test.tsx` 10건(컴포넌트 단위, vitest)과 `e2e/accessibility.spec.ts` 5건(화면 단위, Playwright)이다. CI e2e 잡에 붙였다.
+검사가 실제로 잡은 결함과 조치:
+* 색 대비 7건. 링크 2.96, 로그인 안내 2.76(`opacity: 0.7` 이 원인), BLOCK 라벨 3.14, 보조 텍스트 2.56 x 3. `--color-link` 를 `#1D4ED8`, `--color-block` 을 `#A16207` 로 바꾸고 하드코딩 `#94A3B8` 을 `--text-secondary` 토큰으로 옮겼다. `opacity` 로 흐리게 하던 자리는 색으로만 톤을 낮췔다.
+* 이름 없는 요소 5건. 프로젝트 선택기와 행 수 선택기(`select` 2종), 테이블 체크박스 2건, 다크모드 토글. 토글은 접근 가능한 이름이 "🌙" 였다. 전부 `aria-label` 을 붙였다.
+* 라벨 미연결 2건. 로그인 폼과 강제 비밀번호 변경 화면. `htmlFor`/`id` 로 이었다.
+* 모달 역할 1건. 비밀번호 변경 모달에 `role="dialog"`, `aria-modal`, `aria-labelledby` 를 붙였다.
+* 키보드 함정 1건. 검색 드롭다운을 Escape 로 닫는 핸들러가 아예 없었다. 넣었다.
+확인: 로그인·회원가입·프로젝트 목록·TC 관리 네 화면 모두 serious 이상 0건.
+완료 조건 대조:
+- [X] axe-core 검사가 로그인·프로젝트 목록·TC 관리를 검사한다(회원가입까지 네 화면)
+- [X] serious 이상 위반 0 건
+- [X] CI e2e 잡에서 함께 돌아간다
+- [X] 검사가 실제로 위반을 잡는지 일부러 깨뜨려 확인한다(라벨 없는 input 을 넣어 검출되는 것을 테스트로 고정)
+범위에서 뺀 것은 그대로다. ag-grid 가 스스로 만드는 헤더와 스크롤 동일본은 검사에서 제외했다. 다만 `.ag-root-wrapper` 를 통째로 빼면 그 안의 셀 렌더러까지 같이 빠지므로, 뻐대만 제외하고 셀 내용은 검사에 남겨 두었다.</t>
+        </is>
+      </c>
       <c r="P212" t="inlineStr">
         <is>
           <t>- WCAG AAA 대응
@@ -17168,9 +17217,14 @@
           <t>FE 1.5.4.0</t>
         </is>
       </c>
+      <c r="S212" t="inlineStr">
+        <is>
+          <t>* FE 1.6.0.0 (커밋: a8d2063)</t>
+        </is>
+      </c>
       <c r="T212" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U212" t="inlineStr">
@@ -17236,6 +17290,26 @@
 - QA 엔지니어의 공개 레포에서 가장 먼저 지적받는 안티패턴이다.</t>
         </is>
       </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>회귀 스펙 6개의 `waitForTimeout` 82건을 전부 없았다(현재 0건). 응답 대기(`waitForResponse`)와 상태 단언(web-first assertion)으로 바꿨다.
+그 과정에서 드러난 것이 더 큰 수확이다. **단언이 없거나 조건부로 건너뛰던 테스트 12건**이 있었다. 클릭하고 500ms 기다리고 끝나거나, `try/catch` 로 전부 삼키고 `expect(true).toBe(true)` 로 끝나는 것들이다. 기능이 통째로 고장 나도 통과한다. 전부 실제 검증을 넣었다.
+* 헤더 검색 2건: 1자면 서버를 부르지 않고, 2자 이상이면 부르는지를 응답으로 확인
+* Escape: 드롭다운이 실제로 닫히는지. 기능 자체가 없어 함께 구현했다([SYM-101](https://linear.app/sym804/issue/SYM-101/enh-049-접근성-속성이-없어-스크린리더로-쓸-수-없다))
+* 수행 탭·대시보드 탭: 해당 화면 요소가 뜨는지
+* 검색 하이라이트: `mark.search-hl` 이 붙는지
+* 셀 편집: 저장 응답을 받고 값이 남는지
+* 선택 삭제·복제: 조건부 분기를 없애고 행 수 변화를 단언
+* 404: catch-all 라우트가 `/projects` 로 보내는지
+같이 발견한 것:
+* `test_private_accessible_after_member_add` 가 viewer 를 멤버로 넣고 정리하지 않아, 뒤에 오는 테스트가 순서에 의존한다. 새 권한 테스트는 자기만의 비멤버 계정과 프로젝트를 쓰도록 독립시켰다.
+* ag-grid 체크박스 래퍼(`.ag-selection-checkbox`)를 누르면 포커스만 가고 체크가 안 걸리는 경우가 있다. 실제 `input` 을 `check()` 해야 한다.
+완료 조건 대조:
+- [X] 회귀 스펙 6개의 `waitForTimeout` 제거(82 -&gt; 0)
+- [X] E2E 통과(94 passed). 남은 3건은 `test.skip(CI)` 가 걸린 데이터 의존 테스트로 CI 에서는 건너뛴다
+- [X] 캡처 전용 스펙은 그대로 두었다(66건)</t>
+        </is>
+      </c>
       <c r="P213" t="inlineStr">
         <is>
           <t>- 캡처 전용 스펙(capture-*.spec.ts)의 고정 대기
@@ -17247,9 +17321,14 @@
           <t>FE 1.5.4.0</t>
         </is>
       </c>
+      <c r="S213" t="inlineStr">
+        <is>
+          <t>* FE 1.6.0.0 (커밋: a8d2063)</t>
+        </is>
+      </c>
       <c r="T213" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U213" t="inlineStr">
@@ -17330,14 +17409,40 @@
           <t>- 코드 리뷰 (접근성 작업 중 QA 교차 검증에서 발견)</t>
         </is>
       </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>원인: * `frontend/tsconfig.json` 은 `{"files": [], "references": [...]}` 다. 프로젝트 참조만 들고 있고 자기 파일은 없다.
+* `tsc --noEmit` 은 참조를 타지 않고 그 빈 프로젝트만 본다. 검사 대상이 0 개라 항상 종료코드 0 이다.
+* 실제 컴파일은 `npm run build` 안의 `tsc -b` 가 한다. 그래서 빌드 단계에서야 깨졌다.
+수정 내용: * `.github/workflows/ci.yml` 의 타입 검사 단계를 `npx tsc -b --force` 로 바꿔다.
+* 왜 그런지를 워크플로 주석에 남겨, 다음 사람이 `--noEmit` 으로 되돌리지 않게 했다.</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>* 별도 테스트를 붙이지 않았다. 게이트 자체가 바뀜 것이라, 이제 타입 오류가 있으면 CI 의 해당 단계가 멈춘다.
+* 이번 변경에서 실제로 잡혔다. 새 접근성 테스트가 `ChangePasswordModal` 에 없는 props 를 넘겨 TS2322 가 났고, `--noEmit` 은 그것을 통과시켰다.</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>* CI frontend 잡의 타입 검사 단계. 이제 실제로 검사한다.
+* v1.5.5.1 의 "프로덕션 빌드가 깨지던 타입 오류" 가 이 구멍으로 새어나간 건이다.</t>
+        </is>
+      </c>
       <c r="R214" t="inlineStr">
         <is>
           <t>FE 1.5.5.0</t>
         </is>
       </c>
+      <c r="S214" t="inlineStr">
+        <is>
+          <t>* FE 1.6.0.0 (커밋: a8d2063)</t>
+        </is>
+      </c>
       <c r="T214" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U214" t="inlineStr">

</xml_diff>

<commit_message>
fix(version): 감시 밖에 있던 package-lock 버전 사본 (v1.6.0.1, SYM-104)
package-lock.json 의 version 이 1.5.5.0 에 멈춰 있었다. 나머지 사본 넷은
test_version_consistency.py 가 막고 있어 전부 1.6.0.0 으로 맞아 있었고,
감시 목록에 없던 lock 만 어긋났다.

lock 의 version 은 npm 이 그 시점 package.json 을 박제하는 값이라
"install 먼저, 버전 업 나중" 순서면 한 발 뒤처진 채 커밋된다.
커밋 cfa6316(System v1.5.5.0)부터 벌어졌고 10f10d8 에서 의존성 수정으로
install 이 돌아 한 번 맞았다가 6d19b9c 에서 재발했다.

- lock 의 version 두 자리(최상위, packages[""])를 정본과 맞춤
- 대조 테스트에 lock 케이스 추가. 감시 사본 4곳 -> 5곳
- rules/versioning.md 에 사본 위치와 install 순서 명시
- rules/release_process.md 체크리스트에 사본 갱신·대조 통과 2항목 추가
- 이력 표가 자동 검증 대상이 아님을 명시(SYM-105 로 분리)

QA 2인 통과. lock 의 두 자리를 각각 깨뜨려 테스트 이빨 확인.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U214"/>
+  <dimension ref="A1:U216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -17451,6 +17451,179 @@
         </is>
       </c>
     </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>BUG-144</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>package-lock.json 의 버전만 다른 사본과 어긋난다</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>- frontend/package-lock.json 의 version 이 1.5.5.0 인데 나머지 버전 사본 넷은 1.6.0.0 이다.
+- 어긋난 자리는 lock 파일 안에서 둘이다. 최상위 version(3행)과 packages[""] 의 version(9행).</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>- 릴리즈 노트 '현재 버전' 블록의 Frontend 값과 lock 의 version 두 자리가 같아야 한다.</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>- lock 만 1.5.5.0 에 남았다. backend/main.py, frontend/package.json, i18n ko/en common.json 넷은 1.6.0.0 으로 정상이었다.</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>1. main 브랜치를 체크아웃한다(v1.6.0.0, 커밋 53ed150).
+2. Release_note.md 의 '현재 버전' 블록에서 Frontend 값을 읽는다.
+3. frontend/package-lock.json 의 3행과 9행 version 을 읽는다.
+4. 두 값을 비교한다.</t>
+        </is>
+      </c>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>- git log -L3,3:frontend/package-lock.json 으로 본 lock 버전 이력. 8f3d726(v1.4.0.1)까지 일치, cfa6316(v1.5.3.0)부터 벌어짐, 10f10d8 에서 npm install 이 돌아 우연히 일치, 6d19b9c(v1.5.7.0)에서 재차 벌어짐.
+- 커밋 a8d2063 의 lock diff 는 1.5.4.0 -&gt; 1.5.5.0 인데 같은 커밋의 package.json 은 1.6.0.0 이다. install 이 버전 업보다 먼저 돈 증거다.</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>FE 1.6.0.0</t>
+        </is>
+      </c>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>SYM-104</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>BUG-145</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>rules/versioning.md 의 버전 이력 표가 릴리즈 절반만 담고 있다</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>- rules/versioning.md 의 '현재 버전 이력' 표에 릴리즈 노트 절 44개 중 22개가 없다.
+- 표의 마지막 행은 v1.4.0.1 이고 그 뒤 13개 릴리즈가 반영되지 않았다. 초기 구간(0.1.0.0~0.4.1.0)과 1.2.2.0, 1.2.3.0 도 빠져 있다.</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>- 표가 릴리즈 노트와 같은 릴리즈 집합을 담거나, 담지 않는다면 그 사실이 문서에 명시되어야 한다.</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>- 표는 자동 검증 대상이 아니어서 조용히 벌어졌다. SYM-104 로 lock 사본을 감시 안에 넣었지만 이 표는 여전히 감시 밖이다.</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>1. Release_note.md 에서 '^## v' 로 시작하는 절을 센다.
+2. rules/versioning.md 의 '현재 버전 이력' 표 행을 센다.
+3. 두 집합의 차집합을 구한다.</t>
+        </is>
+      </c>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>- 2026-09-18 실측. 릴리즈 노트 절 44개, 이력 표 22개. 차집합 22건.
+- 빠진 목록: 0.1.0.0 0.2.0.0 0.2.1.0 0.2.1.1 0.3.0.0 0.4.0.0 0.4.1.0 1.2.2.0 1.2.3.0 1.4.1.0 1.5.0.0 1.5.1.0 1.5.1.1 1.5.2.0 1.5.3.0 1.5.4.0 1.5.5.0 1.5.5.1 1.5.6.0 1.5.7.0 1.6.0.0 1.6.0.1</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰. SYM-104 교차 검증 중 QA2 가 지적</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>System 1.6.0.1</t>
+        </is>
+      </c>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>SYM-105</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(log): 이슈 로그 종결 칸 동기화 (SYM-104)
원인 및 수정, 재발 방지, 영향 범위, 수정 버전을 채우고 상태를 완료로 바꿨다.
증거 칸의 System 축과 Frontend 축 혼동도 커밋 해시 기준으로 정정했다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -17513,7 +17513,7 @@
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>- git log -L3,3:frontend/package-lock.json 으로 본 lock 버전 이력. 8f3d726(v1.4.0.1)까지 일치, cfa6316(v1.5.3.0)부터 벌어짐, 10f10d8 에서 npm install 이 돌아 우연히 일치, 6d19b9c(v1.5.7.0)에서 재차 벌어짐.
+          <t>- git log -L3,3:frontend/package-lock.json 으로 본 lock 버전 이력. 8f3d726(v1.4.0.1)까지 일치, cfa6316(System v1.5.5.0, FE 1.5.3.0)부터 벌어짐, 10f10d8 에서 npm install 이 돌아 우연히 일치, 6d19b9c(System v1.5.7.0)에서 재차 벌어짐. v1.5.7.0 의 첫 커밋 10f10d8 은 오히려 일치했던 지점.
 - 커밋 a8d2063 의 lock diff 는 1.5.4.0 -&gt; 1.5.5.0 인데 같은 커밋의 package.json 은 1.6.0.0 이다. install 이 버전 업보다 먼저 돈 증거다.</t>
         </is>
       </c>
@@ -17522,14 +17522,39 @@
           <t>- 코드 리뷰</t>
         </is>
       </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>- 원인: 대조 테스트 test_version_consistency.py 의 감시 목록에 package-lock.json 이 없었다. 감시 안의 사본 넷은 맞아 있었고 감시 밖의 lock 만 어긋났다. lock 의 version 은 npm 이 그 시점 package.json 을 박제하는 값이라 install 을 버전 업보다 먼저 돌리면 옛 값이 박힌다.
+- 수정: lock 의 version 두 자리를 정본과 맞추고, 대조 테스트에 lock 케이스를 추가했다(감시 4곳 -&gt; 5곳).</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>- test_version_consistency.py 에 lock 두 자리를 각각 단언하는 케이스 추가. 각 자리를 따로 깨뜨려 실패하는 것까지 확인했다.
+- rules/versioning.md 에 사본 다섯 곳의 위치와 '버전 업 후 npm install' 순서 명시.
+- rules/release_process.md 체크리스트에 사본 갱신과 대조 통과 확인 2항목 추가.
+- 처음에는 skills/release.md 를 고쳤으나 그 경로는 .gitignore 의 /skills/ 로 추적되지 않아 rules/ 로 옮겼다(QA1 지적).</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>- 버전 표기만. 의존성 트리는 무변경(lock diff 2줄, 380개 패키지 항목·resolved·integrity 그대로).
+- 화면 푸터와 백엔드 앱 버전이 1.6.0.1 로 표시된다.</t>
+        </is>
+      </c>
       <c r="R215" t="inlineStr">
         <is>
           <t>FE 1.6.0.0</t>
         </is>
       </c>
+      <c r="S215" t="inlineStr">
+        <is>
+          <t>FE 1.6.0.1 (커밋: a1c1dd9)</t>
+        </is>
+      </c>
       <c r="T215" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U215" t="inlineStr">

</xml_diff>

<commit_message>
fix(docs): 정본과 어긋난 버전 문서 사본 제거 (v1.6.1.0, SYM-105~107)
버전 판정 기준이 세 곳에 흩어져 있었고 서로 달랐다. 그중 하나는 정본과
반대되는 판정을 지시했다.

- 릴리즈 노트 상단 "버전 체계" 표 제거. 자리 이름이 major/minor 로 정본과
  달랐고 system 을 "대규모 리팩토링"으로 규정해 정본의 "리팩토링은 B 다"
  와 반대를 지시했다 (SYM-107)
- rules/versioning.md 의 이력 표 제거. 릴리즈 노트 절 44개 중 22개가 빠져
  있었고 v0.5.0.0 의 Database 값이 릴리즈 노트와 달랐다. 표에만 있던
  릴리즈는 0건이라 지워도 잃는 것이 없다 (SYM-105)
- 분량 상한이 "- " 항목 줄을 센다는 것을 명시
- 트래커 표기를 Linear 로, git push origin master 를 main 으로 정정

작업 중 낸 사고도 함께 기록한다. 이력 표를 지우며 범위를 "## 현재 버전
이력" 부터 "## 기록 위치" 까지로 잡는 바람에 그 사이에 있던 "버전 사본
위치" 절 22줄이 같이 지워졌다. 직전 커밋에서 추출해 복구했다 (SYM-106)

QA 2인 통과. QA1 이 SYM-106 을, QA2 가 SYM-107 을 잡았다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U216"/>
+  <dimension ref="A1:U218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -17649,6 +17649,181 @@
         </is>
       </c>
     </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>BUG-146</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>문서 절을 범위로 대체하다 사이에 낀 절을 같이 지웠다</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>- rules/versioning.md 에서 '현재 버전 이력' 표를 지우면서 바로 아래 있던 '버전 사본 위치' 절이 함께 사라졌다.
+- 그 절은 직전 커밋 a1c1dd9 에서 SYM-104 재발 방지로 추가한 것이다. 사본 다섯 곳의 위치와 ' 버전 업 후 npm install' 순서를 담고 있었다.</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>- 이력 표만 제거되고 다른 절은 그대로 남아야 한다.</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>- 22줄짜리 절이 통째로 삭제됐다. rules/release_process.md 의 체크리스트가 가리키는 대상이 사라져 참조가 끊겼다.</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>1. 파일에서 '## A' 절을 지우려고 s.index('## A') 부터 s.index('## C') 까지를 범위로 잡는다.
+2. A 와 C 사이에 B 절이 있는지 확인하지 않는다.
+3. 그 구간을 새 내용으로 대체한다.
+4. B 절이 함께 사라진다.</t>
+        </is>
+      </c>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>- 절 목록 대조. 삭제 후 rules/versioning.md 의 '## ' 헤딩은 6개였고 '## 버전 사본 위치' 가 없었다. 복구 후 7개.
+- git show HEAD:rules/versioning.md 로 직전 커밋에서 22줄 절을 그대로 추출해 복구했다.</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰. QA1(Codex)이 rules/release_process.md 의 참조가 끊겼다고 지적</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>System 1.6.0.2</t>
+        </is>
+      </c>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>SYM-106</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>BUG-147</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>릴리즈 노트의 버전 체계 표가 정본과 반대되는 판정을 지시한다</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>- Release_note.md 상단 '버전 체계' 절이 rules/versioning.md 와 다른 내용을 담고 있었다.
+- 자리 이름이 달랐다. 릴리즈 노트는 system.feature.major.minor, 정본은 system.feature.fix.patch.
+- system 자리 정의가 정반대였다. 릴리즈 노트는 '대규모 리팩토링'을 system 으로 규정하는데 정본은 '리팩토링은 B 다. A 가 아니다' 로 못박고 있다.</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>- 버전 자리 판정 기준은 한 곳에만 있어야 한다. 정본은 rules/versioning.md 다.</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>- 파일 맨 앞, 어떤 릴리즈 절보다 먼저 읽히는 자리에 정본과 반대되는 지시가 있었다. 이 표를 보고 판정하면 리팩토링에 A 자리를 올리게 된다.</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>1. Release_note.md 5행 '### 형식' 표의 major/minor 행을 읽는다.
+2. rules/versioning.md 3행 '## 버전 체계' 표의 fix/patch 행을 읽는다.
+3. 자리 이름과 system 자리의 정의를 비교한다.</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>- Release_note.md:5 '### 형식: system.feature.major.minor', system 기준 '대규모 리팩토링, 아키텍처 변경, 하위 호환 불가'.
+- rules/versioning.md:3 '## 버전 체계: system.feature.fix.patch', 그리고 17행 '리팩토링은 B 다. A 가 아니다. 내부 구조만 바꾼 것은 아무리 커도 B 다'.
+- 같은 유형의 실제 피해 사례가 다른 프로젝트에 있다. 전역 규칙에 'A=리팩토링' 이 잘못 적힌 채 굳어 refactor 8개 절 중 A 를 올린 것이 1개뿐이었고 24일 만에 6.0 에서 6.34 가 됐다.</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰. SYM-105 교차 검증 중 QA2 가 지적</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>System 1.6.0.2</t>
+        </is>
+      </c>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>SYM-107</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(log): 이슈 로그 종결 칸 동기화 (SYM-105~107)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -17633,14 +17633,36 @@
           <t>- 코드 리뷰. SYM-104 교차 검증 중 QA2 가 지적</t>
         </is>
       </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>- 원인: 릴리즈별 컴포넌트 버전을 rules/versioning.md 이력 표와 Release_note.md 각 절이 이중으로 들고 있었다. 표는 자동 검증 대상이 아니라 조용히 벌어졌다.
+- 수정: 표를 제거하고 릴리즈 노트 각 절의 컴포넌트 버전 표를 정본으로 가리켰다.</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>- 감시를 늘리는 대신 사본을 없앴다. 지우기 전에 표 22행이 전부 릴리즈 노트에 있는지 전수 대조했고 표에만 있던 릴리즈는 0건이었다.
+- 하지 않을 것: 표를 테스트로 감시하는 방안은 택하지 않았다. 사본을 유지하는 비용이 남는다.</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>- 문서만. rules/versioning.md 의 이력 표 1개.</t>
+        </is>
+      </c>
       <c r="R216" t="inlineStr">
         <is>
           <t>System 1.6.0.1</t>
         </is>
       </c>
+      <c r="S216" t="inlineStr">
+        <is>
+          <t>System 1.6.1.0 (커밋: c1f564c)</t>
+        </is>
+      </c>
       <c r="T216" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U216" t="inlineStr">
@@ -17720,14 +17742,36 @@
           <t>- 코드 리뷰. QA1(Codex)이 rules/release_process.md 의 참조가 끊겼다고 지적</t>
         </is>
       </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>- 원인: 이력 표를 지우며 '## 현재 버전 이력' 부터 '## 기록 위치' 까지를 범위로 잡아 대체했다. 그 사이에 직전 커밋에서 추가한 '## 버전 사본 위치' 절이 끼어 있었다.
+- 수정: git show HEAD:rules/versioning.md 에서 22줄 절을 그대로 추출해 복구했다.</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>- 구간을 범위로 대체할 때는 그 구간에 든 '## ' 절을 먼저 세어 예상과 일치하는지 단언한다. 같은 작업의 다음 삭제(SYM-107)에 이 검사를 적용해 통과했다.
+- 절 목록(grep '^## ')을 작업 전후로 비교한다. 삭제 후 6개, 복구 후 7개로 확인했다.</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>- 커밋 전에 발견해 복구했다. 푸시된 적 없다.</t>
+        </is>
+      </c>
       <c r="R217" t="inlineStr">
         <is>
           <t>System 1.6.0.2</t>
         </is>
       </c>
+      <c r="S217" t="inlineStr">
+        <is>
+          <t>System 1.6.1.0 (커밋: c1f564c)</t>
+        </is>
+      </c>
       <c r="T217" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U217" t="inlineStr">
@@ -17808,14 +17852,36 @@
           <t>- 코드 리뷰. SYM-105 교차 검증 중 QA2 가 지적</t>
         </is>
       </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>- 원인: 버전 판정 기준이 Release_note.md 상단과 rules/versioning.md 두 곳에 있었고 내용이 갈라졌다. 릴리즈 노트 쪽이 자리 이름을 major/minor 로 쓰고 system 을 '대규모 리팩토링' 으로 규정해, 정본의 '리팩토링은 B 다. A 가 아니다' 와 반대를 지시했다.
+- 수정: 릴리즈 노트 상단 표를 제거하고 rules/versioning.md 를 정본으로 가리켰다.</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>- 판정 기준을 한 곳으로 줄였다. 사본이 없으면 갈라질 수 없다.
+- 지운 자리에 무엇이 왜 있었는지 남겨, 다시 만들지 않도록 했다.</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>- 문서만. 다만 이 표를 보고 판정했다면 리팩토링에 A 자리를 올렸을 것이다. 다른 프로젝트에서 같은 오류로 24일 만에 6.0 이 6.34 가 된 사례가 있다.</t>
+        </is>
+      </c>
       <c r="R218" t="inlineStr">
         <is>
           <t>System 1.6.0.2</t>
         </is>
       </c>
+      <c r="S218" t="inlineStr">
+        <is>
+          <t>System 1.6.1.0 (커밋: c1f564c)</t>
+        </is>
+      </c>
       <c r="T218" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U218" t="inlineStr">

</xml_diff>

<commit_message>
feat(run): 테스트 수행 화면에 사전조건 열 (v1.6.2.0, SYM-108)
사전조건은 실행 직전에 갖춰야 하는 상태라 수행자가 봐야 한다. 그런데 TC 관리
화면에만 있어서 수행 중에 화면을 옮겨다녀야 했다.

조사에서 셋을 배제했다. 프로젝트 설정으로 숨긴 것이 아니고(수행 그리드는
field_config 를 읽지 않는다), 회귀도 아니며(그 파일에 precondition 이 있었던
적이 없다), 데이터는 API 응답에 담겨 오고 있었다. 컬럼 정의가 없었을 뿐이다.

- 수행 그리드에 읽기 전용 열 추가. 참조는 PreconditionCell 툴팁으로 펼친다
- 참조 색인은 런의 results 로 만든다. 없으면 안내 문구가 뜬다
- 런 엑셀과 리포트 엑셀에 같은 열 추가. 두 파일의 TC 열 집합을 계약으로 묶었다
- 런 엑셀 col_widths 가 헤더보다 하나 적어 폭이 밀리던 것 수정
- 리포트의 결과 색칠이 열 번호를 박아 쓰던 것을 헤더 이름 기준으로 변경

QA 2인 통과. QA1 이 col_widths 밀림을, QA2 가 리포트 엑셀 누락을 잡았다.
이빨 확인에서 테스트 구멍을 둘 찾아 메웠다. load_only 를 빼도 지연 로딩으로
값이 나와 못 잡던 것은 조회 횟수 비교로, col_widths 밀림은 openpyxl 이 기본
폭을 돌려줘 못 잡던 것은 폭의 성질 비교로 바꿨다.

잔여 누락은 SYM-109(Platform), SYM-110(Ctrl+D), SYM-111(필드 설정)로 분리했다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U218"/>
+  <dimension ref="A1:U222"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -17890,6 +17890,363 @@
         </is>
       </c>
     </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>ENH-051</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>테스트 수행 화면에 사전조건 열 추가</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>- 수행 화면이 보여주는 TC 필드는 no, tc_id, category, depth1, depth2, priority, test_steps, expected_result 여덟이다. precondition 은 columnDefs 에 없다.
+- 설정 문제가 아니다. TestRunManager 는 field_config 를 읽지 않아 프로젝트 설정의 필드 표시 설정이 이 화면에 적용되지 않는다.
+- 회귀가 아니다. git log -S precondition 으로 확인한 결과 이 파일에 precondition 이 있었던 적이 없다.
+- API 응답에는 담겨 온다. TestResultResponse.test_case 가 TestCaseResponse 이고 거기에 precondition 이 있다.
+- 런 엑셀 내보내기도 같다. headers 에 없고 load_only 에도 없어 아예 로드하지 않는다.</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>- 수행 화면에서 사전조건을 읽을 수 있다. 수행자가 TC 관리 화면을 따로 열지 않아도 된다.
+- 다른 TC 를 참조하는 사전조건은 툴팁으로 펼쳐 보인다.
+- 런 엑셀 내보내기에도 같은 열이 실린다.</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>- [ ] 수행 화면에 사전조건 열이 보인다
+- [ ] 그 열은 읽기 전용이다. 수행 중 TC 원문이 고쳐지지 않는다
+- [ ] 참조 형태로 쓴 사전조건이 툴팁에서 펼쳐진다
+- [ ] 런 엑셀 내보내기에 사전조건 열이 실린다
+- [ ] 위를 검증하는 테스트가 있고, 일부러 깨뜨리면 실패한다</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>- 사전조건은 실행 직전에 갖춰야 하는 상태라 수행자가 봐야 하는 정보다. Steps 와 Expected 를 보여주면서 이것만 빼면 수행 중에 화면을 옮겨다녀야 한다.
+- 이 프로젝트는 사전조건을 비중 있게 다룬다. 전용 렌더러 PreconditionCell, 참조 풀이 precondition_service, TC 내보내기의 셀 메모까지 있는데 정작 가장 필요한 화면에만 없다.</t>
+        </is>
+      </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>- TestRunManager 의 columnDefs 에 precondition 이 없었다. 설정 문제도 회귀도 아니고 처음부터 없었다. API 응답에는 담겨 오고 있었다.
+- 수행 그리드에 읽기 전용 열을 넣고 PreconditionCell 을 재사용해 참조를 툴팁으로 펼쳤다. 색인은 런의 results 로 만든다.
+- 런 엑셀(routes/testruns.py)과 리포트 엑셀(routes/reports.py) 양쪽에 같은 열을 넣었다. 리포트는 QA2 가 빠진 것을 잡았다.
+- 부수 수정: 런 엑셀 col_widths 가 헤더보다 하나 적어 폭이 밀리던 것(QA1 지적), 리포트의 결과 색칠이 열 번호를 박아 쓰던 것.</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>- GridEditorContract.test.tsx 에 계약 7건. 이 파일은 '두 그리드 중 한쪽만 고쳐 온 이력' 을 막으려고 만든 자리다.
+- tests_unit/test_run_export_columns.py 13건. 두 엑셀의 TC 열 집합이 같은지 묶었다.
+- 이빨 확인에서 두 번 구멍을 찾아 메웠다. load_only 를 빼도 지연 로딩으로 값이 나와 못 잡던 것은 조회 횟수 비교로, col_widths 밀림은 openpyxl 이 기본 폭을 돌려줘 못 잡던 것을 폭의 성질 비교로 바꿨다.
+- test_export_formula_injection.py 픽스처에 precondition 을 태웠다. 값이 없으면 전 셀을 훑어도 그 열은 검사되지 않는다.
+- 하지 않을 것: 수행 화면에서 사전조건 편집, 셀 안 참조 펼침, 프로젝트 전체 TC 를 색인용으로 추가 조회.</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>- 수행 화면에 열 하나 추가(읽기 전용). 런 엑셀과 리포트 엑셀 열 하나 추가.
+- 되가져오기는 import_service 에 Precondition 매핑이 이미 있어 그대로 들어간다.
+- 잔여 누락은 SYM-109(Platform), SYM-110(Ctrl+D 거짓 성공), SYM-111(필드 표시 설정 미적용)로 분리했다.</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
+        <is>
+          <t>System 1.6.1.0</t>
+        </is>
+      </c>
+      <c r="S219" t="inlineStr">
+        <is>
+          <t>FE 1.6.1.0 / BE 1.6.1.0 (System 1.6.2.0)</t>
+        </is>
+      </c>
+      <c r="T219" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U219" t="inlineStr">
+        <is>
+          <t>SYM-108</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>ENH-052</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>테스트 수행 화면과 런 엑셀에 Platform(test_type) 열 추가</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>- test_type(Platform)이 TC 그리드에 있고(TestCaseGrid.tsx:395) TC 목록 엑셀에도 있고(export_service.py:87) 프로젝트 설정에 숨김 가능 필드로 등록돼 있는데(ProjectSettings.tsx:397), 수행 화면과 런 엑셀에는 없다.
+- SYM-108 의 사전조건과 정확히 같은 모양의 누락이다.
+- 함께 빠진 것은 TestCase.remarks 와 custom_fields 다. 수행 그리드의 Remarks 열은 TestResult.remarks 라 이름만 같고 다른 값이다. r1~r3 은 TC 그리드에도 없는 레거시라 제외한다.</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>- 수행자가 그 TC 가 Web 인지 Android 인지 화면에서 확인할 수 있다.
+- 런 엑셀과 리포트 엑셀에도 같은 열이 실린다.</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>- [ ] 수행 화면에 Platform 열이 보이고 읽기 전용이다
+- [ ] 런 엑셀과 리포트 엑셀에 같은 열이 실린다
+- [ ] GridEditorContract 에 계약 테스트가 있다
+- [ ] TestCase.remarks 를 넣을지 뺄지 결정하고 근거를 남긴다</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>- SYM-108 을 고치며 같은 유형의 누락이 남아 있음을 확인했다. 지금 적어 두지 않으면 다음에 또 제보로 발견된다.
+- 수행 플랫폼은 실행 방법을 가르는 정보라 사전조건만큼 수행에 직접 쓰인다.</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>- r1~r3 은 넣지 않는다. TC 그리드에도 없는 레거시 칼럼이다.</t>
+        </is>
+      </c>
+      <c r="R220" t="inlineStr">
+        <is>
+          <t>System 1.6.1.0</t>
+        </is>
+      </c>
+      <c r="T220" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U220" t="inlineStr">
+        <is>
+          <t>SYM-109</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>BUG-148</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>trivial</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Ctrl+D 가 읽기 전용 TC 열에서 채웠다고 알린다</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>- 수행 그리드에서 읽기 전용 TC 열(category, test_steps, precondition 등 8개)에 Ctrl+D 를 누르면 '몇 건 채웠다' 토스트가 뜨고 저장 요청이 나간다.
+- 실제로는 아무것도 바뀌지 않는다.</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>- 편집할 수 없는 열에서는 Ctrl+D 가 아무 일도 하지 않고 토스트도 뜨지 않아야 한다.</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>- TestRunManager.tsx:459-476 에서 node.data[field] = sourceValue 를 하는데 field 가 'test_case.precondition' 같은 점 찍힌 경로다. 중첩 객체가 아니라 평평한 문자열 키가 새로 생겨 화면 값은 그대로다.
+- 저장 요청은 test_case_id/result/actual_result/issue_link/remarks/duration_sec 화이트리스트라 TC 원문이 새지는 않는다.</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>- 수행 그리드에 행이 둘 이상 있고 첫 행이 선택돼 있다.</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>1. 테스트 수행 화면에서 런을 연다.
+2. Category 나 Test Steps 열의 셀을 클릭한다.
+3. 아래 행까지 선택한 뒤 Ctrl+D 를 누른다.
+4. 토스트 문구와 화면 값을 비교한다.</t>
+        </is>
+      </c>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>- TestRunManager.tsx:459-476 의 node.data[field] 대입. field 는 columnDefs 의 field 값이라 test_case 로 시작하는 열은 점 표기다.
+- 저장 경로는 saveOneResult(:384)와 saveManyResults(:160)이고 둘 다 고정 화이트리스트다.</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰. SYM-108 교차 검증 중 QA2 가 지적</t>
+        </is>
+      </c>
+      <c r="R221" t="inlineStr">
+        <is>
+          <t>System 1.6.1.0</t>
+        </is>
+      </c>
+      <c r="T221" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U221" t="inlineStr">
+        <is>
+          <t>SYM-110</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>ENH-053</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>수행 그리드가 프로젝트의 필드 표시 설정을 따르지 않는다</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>- 프로젝트 설정의 기본 필드 설정(표시 여부, 표시 이름)은 TC 그리드에만 적용된다. TestCaseGrid.tsx:344-348 의 fieldDisplay 가 그 일을 한다.
+- 수행 그리드는 field_config 를 읽지 않고 headerName 을 영문으로 박아 둔다.
+- 그래서 필드 이름을 '사전조건 / 테스트 데이터' 로 바꾼 프로젝트에서 두 화면의 헤더가 다르게 보이고, 숨긴 필드가 수행 화면에는 그대로 나온다.</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>- 두 그리드가 같은 설정을 따른다. 이름을 바꾸면 양쪽이 같이 바뀌고, 숨기면 양쪽에서 사라진다.</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>- [ ] 수행 그리드가 project.field_config 의 표시 이름을 반영한다
+- [ ] 숨김으로 둔 필드는 수행 그리드에서도 빠진다
+- [ ] test_steps 와 expected_result 는 canHide:false 라 숨겨지지 않는다
+- [ ] 두 그리드가 같은 설정을 본다는 계약 테스트가 있다</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>- SYM-108 로 숨김 가능 필드(precondition)를 수행 화면에 하나 더 얹었다. 설정과 어긋나는 면이 그만큼 넓어졌다.
+- 제보가 '설정에서 숨긴 것 아니냐' 로 시작했던 만큼 사용자도 두 화면이 같은 설정을 따를 것이라 기대한다.</t>
+        </is>
+      </c>
+      <c r="P222" t="inlineStr">
+        <is>
+          <t>- 수행 전용 열(Result, Actual Result, 첨부, 소요)은 이 설정의 대상이 아니다.</t>
+        </is>
+      </c>
+      <c r="R222" t="inlineStr">
+        <is>
+          <t>System 1.6.1.0</t>
+        </is>
+      </c>
+      <c r="T222" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U222" t="inlineStr">
+        <is>
+          <t>SYM-111</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(run): 수행 화면의 Platform 열과 필드 설정 적용 (v1.6.3.0, SYM-109~111)
SYM-108 교차 검증에서 나온 같은 유형의 잔여 결함 셋을 한꺼번에 고친다.

- 수행 화면과 두 엑셀에 Platform(test_type) 열 추가. 읽기 전용 (SYM-109)
- 수행 그리드가 프로젝트 필드 설정을 따른다. TC 에서 오는 아홉 열만 대상이고
  수행 전용 열은 늘 보인다 (SYM-111)
- Ctrl+D 를 채워도 되는 열로 한정 (SYM-110)

TestCase.remarks 는 넣지 않는다. 수행 그리드의 Remarks 는 TestResult.remarks 라
같은 이름의 열이 둘이 되면 어느 칸에 적을지 헷갈린다. custom_fields 는 동적
컬럼 생성이 필요해 범위를 넘는다. 근거는 코드 주석에 남겼다.

QA 2인 통과. 두 QA 가 같은 곳을 짚었고 첫 수정이 뒤집혔다.

처음에는 Ctrl+D 를 "editable 이 false 면 막는다" 로 고쳤는데 판정이 반대로
걸린 것이었다. editable 을 아예 안 쓴 열 아홉은 undefined 라 그대로 통과하고,
정작 Ctrl+D 의 주 용도인 Result 는 커스텀 렌더러 때문에 editable:false 라서
막혔다. 소요(초)는 저장 본문 화이트리스트에 있어 타이머 측정값이 실제로
덮어써지는 경로였다. 채워도 되는 열 화이트리스트로 다시 짰다.

ESLint 가 CI 를 깨는 것도 푸시 전에 잡았다. _key 를 떼는 자리에 TestCaseGrid
에는 있는 disable 주석이 빠져 있었다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -18055,9 +18055,23 @@
 - 수행 플랫폼은 실행 방법을 가르는 정보라 사전조건만큼 수행에 직접 쓰인다.</t>
         </is>
       </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>- SYM-108 과 같은 유형의 누락이었다. TC 그리드와 TC 목록 엑셀에는 있는데 수행 화면과 두 엑셀에만 없었다.
+- 수행 그리드에 읽기 전용 Platform 열을 넣고, 런 엑셀과 리포트 엑셀에도 같은 열을 넣었다.
+- TestCase.remarks 는 넣지 않기로 했다. 수행 그리드에 이미 Remarks 열이 있는데 그것은 TestResult.remarks 라, 같은 이름의 열이 둘이 되면 수행자가 어느 칸에 적을지 헷갈린다. custom_fields 는 동적 컬럼 생성이 필요해 이번 범위를 넘는다. 근거는 TestRunManager.tsx 주석에 남겼다.</t>
+        </is>
+      </c>
       <c r="P220" t="inlineStr">
         <is>
-          <t>- r1~r3 은 넣지 않는다. TC 그리드에도 없는 레거시 칼럼이다.</t>
+          <t>- GridEditorContract 에 Platform 계약 3건. 열 제거 조작에서 4건이 실패하는 것을 확인했다.
+- 리포트 엑셀에도 N+1 회귀 테스트를 걸어 런 엑셀과 대칭을 맞췄다. load_only 에서 test_type 을 빼면 실패한다.
+- 하지 않을 것: r1~r3 은 TC 그리드에도 없는 레거시라 넣지 않았다.</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>- 수행 화면 열 하나, 런 엑셀과 리포트 엑셀 각 열 하나.</t>
         </is>
       </c>
       <c r="R220" t="inlineStr">
@@ -18065,9 +18079,14 @@
           <t>System 1.6.1.0</t>
         </is>
       </c>
+      <c r="S220" t="inlineStr">
+        <is>
+          <t>FE 1.6.2.0 / BE 1.6.2.0 (System 1.6.3.0)</t>
+        </is>
+      </c>
       <c r="T220" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U220" t="inlineStr">
@@ -18153,14 +18172,38 @@
           <t>- 코드 리뷰. SYM-108 교차 검증 중 QA2 가 지적</t>
         </is>
       </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>- 원인: Ctrl+D 가 열을 가리지 않고 node.data[field] 에 대입했다. field 가 'test_case.precondition' 같은 점 찍힌 경로라 중첩이 아니라 평평한 키가 새로 생겨, 화면 값은 그대로인데 토스트가 뜨고 저장 요청이 나갔다.
+- 수정: 채워도 되는 열(result, actual_result, issue_link, remarks)만 통과시킨다.
+- ★처음에는 'editable 이 false 면 막는다' 로 고쳤다가 QA 에서 뒤집혔다. 판정이 반대로 걸린 것이었다. editable 을 아예 안 쓴 열 아홉은 undefined 라 통과하고, 정작 Ctrl+D 의 주 용도인 Result 는 커스텀 렌더러 때문에 editable:false 라서 막혔다.</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>- 테스트 5건. 읽기 전용 TC 열, editable 이 undefined 인 열, 소요(초), Result, 실제 결과를 각각 본다.
+- 테스트 헬퍼가 colDef 를 손으로 만들지 않고 실제 columnDefs 에서 찾아 쓴다. 손으로 만들면 구현과 테스트가 같은 가정을 공유해 undefined 경로를 영영 못 본다.
+- 이빨 확인: 틀린 가드로 되돌리면 3건, 가드를 빼면 3건, 소요(초)를 화이트리스트에 넣으면 1건이 실패한다.</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>- 소요(초) 열에서 Ctrl+D 가 동작하지 않게 됐다. 그 열은 저장 본문 화이트리스트에 있어, 그냥 뒀으면 타이머 측정값이 실제로 덮어써져 저장됐다.</t>
+        </is>
+      </c>
       <c r="R221" t="inlineStr">
         <is>
           <t>System 1.6.1.0</t>
         </is>
       </c>
+      <c r="S221" t="inlineStr">
+        <is>
+          <t>FE 1.6.2.0 / BE 1.6.2.0 (System 1.6.3.0)</t>
+        </is>
+      </c>
       <c r="T221" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U221" t="inlineStr">
@@ -18226,9 +18269,21 @@
 - 제보가 '설정에서 숨긴 것 아니냐' 로 시작했던 만큼 사용자도 두 화면이 같은 설정을 따를 것이라 기대한다.</t>
         </is>
       </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>- 원인: field_config 를 TestCaseGrid 만 읽었다. 수행 그리드는 headerName 을 영문으로 박아 두고 숨김도 반영하지 않았다.
+- 수정: TC 그리드와 같은 규칙(_key + fieldDisplay)을 수행 그리드에 적용했다. 대상은 TC 에서 오는 아홉 열이다.</t>
+        </is>
+      </c>
       <c r="P222" t="inlineStr">
         <is>
-          <t>- 수행 전용 열(Result, Actual Result, 첨부, 소요)은 이 설정의 대상이 아니다.</t>
+          <t>- 수행 전용 열에는 _key 를 붙이지 않는다. 특히 Remarks 가 위험하다. 이름만 같고 TestResult.remarks 라, 섞였으면 TC 비고를 숨긴 프로젝트에서 수행 결과 비고가 사라져 결과를 못 적는다. 그것을 잡는 테스트를 따로 넣었다.
+- 하지 않을 것: 수행 전용 열(Result, 실제 결과, 첨부, 소요)은 이 설정의 대상이 아니다.</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>- 필드 이름을 바꾼 프로젝트는 수행 화면 헤더도 같이 바뀐다. 숨긴 TC 열은 수행 화면에서도 빠진다. 내보내기 파일에는 그대로 실린다.</t>
         </is>
       </c>
       <c r="R222" t="inlineStr">
@@ -18236,9 +18291,14 @@
           <t>System 1.6.1.0</t>
         </is>
       </c>
+      <c r="S222" t="inlineStr">
+        <is>
+          <t>FE 1.6.2.0 / BE 1.6.2.0 (System 1.6.3.0)</t>
+        </is>
+      </c>
       <c r="T222" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U222" t="inlineStr">

</xml_diff>

<commit_message>
fix(a11y): 다크 테마 명암비가 AA 에 못 미치던 토큰 (v1.6.3.1, SYM-55 SYM-56)
선택 상태 버튼과 탭, 오류 문구가 WCAG AA(4.5:1)에 못 미쳤다. 두 이슈 모두
"검사가 없어서" 남아 있었다. jsdom 이 CSS 변수를 풀어 주지 않아 axe 기반
접근성 테스트로는 토큰 조합을 볼 수 없다.

- 다크 --accent 4.31 -> 4.62, --text-danger 카드 4.42 -> 6.01
- 다크 --color-fail 이 --text-danger 가 퇴출한 값 그대로였다. 배지가 아니라
  ReportView 의 FAIL 건수 등 본문 글자색이다
- 라이트 --text-danger 가 연분홍 경고 배경에서 4.38, --color-na 가 4.47
- 색상과 채도는 두고 명도만 조정해 원래 인상을 유지했다

index.css 를 직접 읽어 상대휘도로 재는 검사를 넣었다. 손으로 관리하는 목록은
또 새므로 인벤토리 단언도 같이 붙였다. --text-* / --color-* 토큰이 검사
목록에도 제외 목록에도 없으면 실패한다. 넣자마자 13개가 샜고 그중 --color-na
가 진짜 미달이었다.

QA 2인 통과. QA2 가 --color-fail 과 연분홍 배경 두 곳을 잡았다.

SYM-39 는 확인해 보니 v1.5.4.0 의 schema_guard 로 이미 해결돼 있었다. 구버전
스키마를 흉내낸 인스펙터로 실제로 막히는 것을 확인하고 이슈만 닫는다.

SYM-51 은 열어 둔다. 자세한 것은 그 이슈에 적었다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -11668,14 +11668,36 @@
           <t>- 코드 리뷰 (SYM-37 QA 교차검증, Codex)</t>
         </is>
       </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>- 이번 릴리즈에서 고친 것이 아니다. 확인해 보니 v1.5.4.0(커밋 37d6363)에서 이미 해결돼 있었고 이슈만 열려 있었다.
+- backend/services/schema_guard.py 의 assert_schema_is_current 가 stamp(head) 전에 표지 컬럼을 검사하고, 없으면 SchemaMismatch 로 기동을 멈춘다. 이슈가 요구한 '어긋난 것을 감지해 기동을 멈추고 알린다' 그대로다.</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_schema_guard.py 4건이 지킨다.
+- 말만 믿지 않고 구버전 스키마(test_runs.sheet_names 없음)를 흉내낸 인스펙터로 직접 호출해 실제로 막히는 것을 확인했다.</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>- 없음. 코드는 이미 들어가 있었다.</t>
+        </is>
+      </c>
       <c r="R153" t="inlineStr">
         <is>
           <t>BE 1.3.3.0</t>
         </is>
       </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>BE 1.5.4.0 (커밋: 37d6363)</t>
+        </is>
+      </c>
       <c r="T153" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U153" t="inlineStr">
@@ -13376,14 +13398,36 @@
           <t>- 코드 리뷰 (SYM-54 교차 검증 중 Codex 지적)</t>
         </is>
       </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>- 원인: 다크 --accent(#4B7BBE)에 흰 글자를 얹는 조합이 4.31:1 로 일반 텍스트 AA(4.5:1)에 못 미쳤다. 프로젝트 탭, 시트 탭, 대시보드 날짜 필터가 모두 이 조합이다.
+- 수정: #4876B6 으로 조정(4.62:1). 색상(H)과 채도(S)는 그대로 두고 명도(V)만 낮춰 원래 인상을 유지했다.</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>- cssTokens.test.ts 에 토큰 명암비 검사 추가. index.css 를 직접 읽어 WCAG 상대휘도로 잰다. jsdom 은 CSS 변수를 안 풀어 주므로 axe 기반 접근성 테스트로는 이 조합을 볼 수 없다.
+- 옛 값으로 되돌리면 실패하는 것을 확인했다.</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>- 다크 테마의 선택 상태 배경색. 전후 차이가 눈에 거의 안 띄는 수준이다.</t>
+        </is>
+      </c>
       <c r="R169" t="inlineStr">
         <is>
           <t>FE 1.5.1.1</t>
         </is>
       </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>FE 1.6.2.1 (System 1.6.3.1)</t>
+        </is>
+      </c>
       <c r="T169" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U169" t="inlineStr">
@@ -13446,9 +13490,24 @@
 - SYM-54 가 추가한 미선언 토큰 검사는 폴백이 있는 참조를 잡지 않으므로 이 자리는 계속 남는다</t>
         </is>
       </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>- 착수해 보니 절반은 이미 돼 있었다. --danger 가 --text-danger 로 바뀌고 라이트/다크 둘 다 선언된 상태였다. 남아 있던 것은 완료 조건 2번(명암비 4.5:1)이다.
+- 다크 --text-danger 가 카드 4.42 입력 4.02 였다. #F87171 로 올렸다(6.01 / 5.46).
+- 교차 검증에서 두 곳이 더 나왔다. 다크 --color-fail 이 퇴출한 #EF4444 그대로였고(배지가 아니라 ReportView 의 FAIL 건수 등 본문 글자색이다), 라이트 --text-danger 가 연분홍 경고 배경에서 4.38 이었다. 둘 다 고쳤다.
+- 검사 목록을 만들다 --color-na 가 라이트에서 4.47 인 것도 찾아 함께 고쳤다.</t>
+        </is>
+      </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>- 폴백 있는 참조 전체를 금지하는 규칙 추가는 이번 범위가 아니다</t>
+          <t>- 명암비 검사에 더해 인벤토리 단언을 넣었다. --text-* / --color-* 토큰이 검사 목록에도 제외 목록에도 없으면 실패한다. 손목록만 두면 또 샌다. 실제로 넣자마자 13개가 샜고 그중 하나가 진짜 미달이었다.
+- 한계를 파일 첫머리에 적었다. 토큰 값이 #RRGGBB 인 것만 읽으므로 rgba() 배경과 하드코딩 색은 대상 밖이다.
+- 하지 않을 것: 폴백 있는 참조 전체를 금지하는 규칙은 이번에도 넣지 않았다.</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>- 라이트와 다크의 오류 문구, FAIL/N-A 건수 글자색.</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
@@ -13456,9 +13515,14 @@
           <t>FE 1.5.1.1</t>
         </is>
       </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>FE 1.6.2.1 (System 1.6.3.1)</t>
+        </is>
+      </c>
       <c r="T170" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U170" t="inlineStr">

</xml_diff>

<commit_message>
feat(run): 테스트 수행 화면 우선순위 멀티 선택 (v1.6.6.0, SYM-113)
Priority 필터를 단일 select 에서 체크박스 드롭다운으로 바꿨다. 고른 값 중
하나라도 맞으면 남고, Result/Category/검색어와는 AND 로 합쳐진다.

- 버튼 라벨은 안 고르면 "전체", 하나면 그 값, 둘 이상이면 개수다
- 우선순위를 비워 둔 TC 가 있으면 목록 맨 아래에 (미지정) 이 생긴다
- 고른 값이 지금 결과 집합에 없어도 목록에 남긴다. 시트를 옮기면 그 값이
  목록에서 빠져 체크를 풀 수단이 없어지고 그리드가 빈 채로 잠겼다
- 바깥 클릭과 Esc 로 닫고, 런이나 시트를 옮기면 열린 드롭다운을 닫는다
- 활성 버튼은 accent 배경에 흰 글자다. accent 를 글자색으로 쓰면 다크에서
  3.27:1 로 AA 에 못 미친다. 이 변수는 흰 글자를 얹는 배경 기준 값이다(SYM-55)

테스트 531건 통과. 훅 단위 12건과 화면 통합 4건이 새로 붙었다.
회귀 체크리스트에 TC-TR-031~033 추가, 사용자 매뉴얼 8-8 절 신설.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U223"/>
+  <dimension ref="A1:U224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -18521,6 +18521,89 @@
         </is>
       </c>
     </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>ENH-054</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>테스트 수행 화면에서 우선순위를 하나만 고를 수 있다</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>- 테스트 수행 화면의 Priority 필터가 단일 select 라 한 번에 한 값만 고른다
+- 핵심과 중요를 같이 보려면 값을 바꿔 가며 두 번 확인해야 한다
+- AG Grid 컬럼 필터는 꺼져 있고, 체크박스형 Set Filter 는 Enterprise 기능이라 community 35.1.0 에서는 쓸 수 없다</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>- 우선순위를 여러 개 함께 고른다. 고른 것 중 하나라도 맞는 행이 남는다
+- 버튼에 고른 값이, 둘 이상이면 개수가 표시된다
+- 우선순위를 비워 둔 TC 가 있으면 (미지정) 선택지가 생겨 그 행만 따로 볼 수 있다</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>- [ ] 우선순위를 여러 개 체크하면 OR 로 걸린다
+- [ ] Result, Category, 검색어와는 AND 로 합쳐진다
+- [ ] 값이 빈 행을 (미지정) 으로 골라낼 수 있다
+- [ ] 시트를 옮겨 고른 값이 그 시트에 없어도 체크를 풀 수 있다
+- [ ] 바깥 클릭과 Esc 로 닫힌다
+- [ ] 다크 테마에서 활성 버튼 명암비가 AA 를 넘는다</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>- 회귀 수행에서 핵심과 중요만 먼저 도는 일이 잦은데, 지금은 두 번 나눠 확인해야 한다
+- 우선순위가 빈 TC 는 어떤 값을 골라도 화면에서 사라지는데 그 사실을 알 방법이 없다</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>- Result 와 Category 의 멀티 선택. 이번 범위는 우선순위만
+- 드롭다운 포커스 트랩. 기존 결과 일괄입력 드롭다운도 없어 따로 다룬다</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
+        <is>
+          <t>FE 1.6.2.1</t>
+        </is>
+      </c>
+      <c r="T224" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U224" t="inlineStr">
+        <is>
+          <t>SYM-113</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(grid): 셀 텍스트 복사 허용, 클릭 한 번에 편집되던 동작 수정 (v1.6.7.0, SYM-114/115/116)
- 두 그리드에서 singleClickEdit 을 뺐다. 클릭 한 번은 셀 선택이고 편집은
  더블클릭·F2·바로 타이핑으로 시작한다. 매뉴얼은 이전부터 더블클릭이라고
  안내하고 있었고 구현만 달랐다
- enableCellTextSelection 과 ensureDomOrder 를 켰다. 절차·기대 결과처럼
  읽기 전용인 열을 포함해 셀 안의 글자를 끌어서 선택해 복사할 수 있다
- 매뉴얼 단축키 표의 Ctrl+C/V 문구를 실제 동작에 맞게 고쳤다(ko/en).
  AG Grid 의 셀 범위 복사는 Enterprise 전용이라 Community 만 쓰는 이
  제품에는 없는데 표에 실려 있었다
- 유닛 계약 테스트와 E2E 를 붙였다. singleClickEdit 을 일부러 되살려
  E2E 가 실패하는 것까지 확인했다

수행 시트의 편집 가능 열은 그대로 셋(실제 결과, 이슈 링크, 비고)이고
TC 원문은 계속 읽기 전용이다.

QA 2인 통과

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U224"/>
+  <dimension ref="A1:U227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -18582,6 +18582,17 @@
 - 우선순위가 빈 TC 는 어떤 값을 골라도 화면에서 사라지는데 그 사실을 알 방법이 없다</t>
         </is>
       </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>* `useResultFilters` 의 `filterPriority`(string) 를 `filterPriorities`(string\[\]) 로 바꾸고 `togglePriority` 를 더했다. 빈 배열이 "전체"다
+* Priority 필터를 체크박스 드롭다운으로 교체했다. 버튼 라벨은 전체 / 고른 값 / 개수 순으로 바뀐다
+* 우선순위가 빈 행이 있을 때만 (미지정) 선택지가 생긴다. 실측으로 이 값이 있는 TC 가 162건 있었다(ymseo_test 160, 런시트범위\_tmp 2)
+* 고른 값이 현재 결과 집합에 없어도 목록에 남긴다. 시트별 우선순위 구성이 달라(stockradar 의 "표면 커버리지 보강" 시트는 중요 하나뿐) 시트를 옮기면 체크를 풀 수단이 사라지고 그리드가 빈 채로 잠겼다
+* 바깥 클릭과 Esc 로 닫고, 런이나 시트를 옮기면 열린 드롭다운을 닫는다
+* 활성 버튼을 accent 배경에 흰 글자로 칠했다. accent 를 글자색으로 쓰면 다크에서 3.27:1 로 AA(4.5:1) 에 못 미쳤다. 이 변수는 흰 글자를 얹는 배경 기준으로 보정된 값이다(4.62:1)
+* 완료 조건과 어긋난 것은 없다</t>
+        </is>
+      </c>
       <c r="P224" t="inlineStr">
         <is>
           <t>- Result 와 Category 의 멀티 선택. 이번 범위는 우선순위만
@@ -18593,14 +18604,327 @@
           <t>FE 1.6.2.1</t>
         </is>
       </c>
+      <c r="S224" t="inlineStr">
+        <is>
+          <t>FE 1.6.3.0 (System 1.6.6.0, 커밋 a35160f)</t>
+        </is>
+      </c>
       <c r="T224" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U224" t="inlineStr">
         <is>
           <t>SYM-113</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>ENH-055</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>테스트 수행 시트에서 셀 텍스트를 끌어서 복사할 수 없다</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>- 셀 안의 글자를 마우스로 끌어도 선택되지 않는다. AG Grid 가 user-select:none 을 걸기 때문이다.
+- 절차·기대 결과·사전조건은 읽기 전용 열인데도 복사가 막혀 있다. 편집도 안 되고 복사도 안 되는 상태다.</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>- 셀 안의 글자를 끌어 선택해 복사할 수 있다.
+- 읽기 전용 열과 편집 가능 열 모두에서 된다.</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>- [x] 두 그리드에서 셀 텍스트를 끌어 선택할 수 있다
+- [x] 읽기 전용 열에서도 선택된다
+- [x] 결과 드롭다운, Shift+클릭 범위 채우기, Ctrl+D 가 그대로 동작한다</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>- 수행자가 절차나 기대 결과를 다른 곳에 옮길 때마다 막힌다. 눈으로 읽고 손으로 옮기는 수밖에 없다.
+- 같은 화면을 매일 쓰는 작업이라 누적 비용이 크다.</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>- 두 그리드에 enableCellTextSelection 과 ensureDomOrder 를 켰다.
+- 브라우저에서 user-select 가 text 로 바뀐 것과 실제로 글자가 선택되는 것을 확인했다.</t>
+        </is>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>- AG Grid 범위 복사(Ctrl+C 로 여러 셀) 는 Enterprise 기능이라 넣지 않는다. Community 에는 없다.</t>
+        </is>
+      </c>
+      <c r="R225" t="inlineStr">
+        <is>
+          <t>FE 1.6.3.0</t>
+        </is>
+      </c>
+      <c r="S225" t="inlineStr">
+        <is>
+          <t>FE 1.6.4.0</t>
+        </is>
+      </c>
+      <c r="T225" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U225" t="inlineStr">
+        <is>
+          <t>SYM-114</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>BUG-150</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>TC 그리드가 클릭 한 번에 편집 모드로 들어간다</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>- TC 관리 그리드에서 셀을 한 번 클릭하면 곧바로 편집기가 열린다.
+- 값을 고칠 생각 없이 내용만 확인하려 해도 편집 상태가 되어, 잘못 누르면 값이 바뀐다.
+- 편집기가 열린 칸은 글자를 끌어서 선택할 수 없다.</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>- 클릭 한 번은 셀 선택까지만 한다.
+- 편집은 더블클릭이나 F2 로 시작한다. 사용자 매뉴얼도 그렇게 안내하고 있다.</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>- 클릭 즉시 인라인 편집기가 열렸다.</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>1. TC 관리 그리드를 연다.
+2. 아무 셀이나 한 번 클릭한다.
+3. 편집기가 열린 것을 확인한다.</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>- 매뉴얼 grid_li1 은 '셀을 더블 클릭하면 인라인 편집 모드로 진입합니다' 라고 적고 있었다(frontend/src/i18n/ko/manual.json:195). 문서가 맞고 구현이 달랐다.
+- 그리드 설정에 singleClickEdit={true} 가 있었다(TestCaseGrid.tsx, TestRunManager.tsx).</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>- 사용자</t>
+        </is>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>원인: - 두 그리드 모두 singleClickEdit 을 켜 두었다. 빠른 입력을 노린 설정으로 보이나 매뉴얼과 어긋났고, 편집기가 열리면 텍스트 선택이 막히는 부작용이 있었다.
+수정 내용: - 두 그리드에서 singleClickEdit 을 제거해 AG Grid 기본값인 더블클릭 편집으로 되돌렸다.
+- 셀 선택 후 바로 타이핑하는 진입은 그대로라 대량 입력의 타수는 늘지 않는다.</t>
+        </is>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>- 유닛 계약 테스트에 두 그리드의 singleClickEdit 이 true 가 아닌지 단언을 넣었다(GridEditorContract.test.tsx).
+- E2E 에 실제 DOM 기준 단일 클릭/더블클릭 검증을 넣었다. singleClickEdit 을 일부러 되살려 그 테스트가 실패하는 것까지 확인했다.</t>
+        </is>
+      </c>
+      <c r="Q226" t="inlineStr">
+        <is>
+          <t>- TC 관리 그리드와 테스트 수행 그리드의 편집 진입 방식.</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>FE 1.6.3.0</t>
+        </is>
+      </c>
+      <c r="S226" t="inlineStr">
+        <is>
+          <t>FE 1.6.4.0</t>
+        </is>
+      </c>
+      <c r="T226" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U226" t="inlineStr">
+        <is>
+          <t>SYM-115</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>BUG-151</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>trivial</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>매뉴얼이 구현되지 않은 Ctrl+C/V 셀 복사 기능을 안내한다</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>- 사용자 매뉴얼 단축키 표에 'Ctrl + C / V = 복사 / 붙여넣기, TC 관리 그리드' 항목이 있다.
+- 그런 기능이 구현되어 있지 않다. 안내를 보고 눌러도 아무 일도 일어나지 않는다.</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>- 매뉴얼은 실제로 되는 것만 적는다.</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>- 되지 않는 조작을 표에 싣고 있었다.</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>1. 운영 매뉴얼의 단축키 표를 연다.
+2. TC 관리 그리드에서 셀을 선택하고 Ctrl+C 를 누른다.
+3. 다른 셀에서 Ctrl+V 를 누른다.</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>- AG Grid 의 셀 범위 복사·붙여넣기는 Enterprise 전용이다. 이 프로젝트는 ag-grid-community 만 쓰고 ClipboardModule 도 LicenseManager 도 없다(등록 모듈은 AllCommunityModule 하나).
+- 앱 코드에도 Ctrl+C 처리가 없다(grep 0건).
+- 브라우저에서 셀에 포커스만 준 채 복사를 시도하면 선택된 글자가 없어 아무것도 복사되지 않는 것을 확인했다.</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰</t>
+        </is>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>원인: - 구현되지 않은 기능이 매뉴얼에 적혀 있었다. 언제 들어갔는지는 확인하지 못했다.
+수정 내용: - 단축키 표 문구를 '끌어서 선택한 글자 복사 / 편집 중 붙여넣기' 로 고치고 적용 위치를 두 그리드로 바로잡았다(ko/en).
+- 그리드 편집 설명에 한 번 클릭은 선택이고 그 상태에서 글자를 끌어 복사할 수 있다는 문장을 넣었다.</t>
+        </is>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>- 붙이지 못했다. 매뉴얼 문구가 실제 동작과 맞는지 기계로 확인할 방법이 없다. 단축키 표 항목마다 대응하는 E2E 를 두는 것이 근본 처방이나 이번 범위를 넘는다.</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>- 사용자 매뉴얼 단축키 표와 그리드 편집 설명(ko, en).</t>
+        </is>
+      </c>
+      <c r="R227" t="inlineStr">
+        <is>
+          <t>FE 1.6.3.0</t>
+        </is>
+      </c>
+      <c r="S227" t="inlineStr">
+        <is>
+          <t>FE 1.6.4.0</t>
+        </is>
+      </c>
+      <c r="T227" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U227" t="inlineStr">
+        <is>
+          <t>SYM-116</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(release): 빠져 있던 릴리즈 태그 34개 소급, 누락 검사 추가 (v1.6.7.1, SYM-117)
rules/release_process.md 는 커밋 뒤에 태그를 달라고 지시하는데 지켜지지 않아
릴리즈 노트 절 52개 중 태그가 7개뿐이었다. v1.2.1.0 이후 45개가 빠져 있었다.

- 커밋 메시지의 버전 표기로 릴리즈 커밋을 찾아 34개를 소급해 달았다.
  v1.2.2.0 과 v0.x 초기 11개는 커밋을 특정하지 못해 달지 않았다.
  틀린 태그는 없는 태그보다 나쁘다
- test_version_consistency.py 가 지난 릴리즈의 태그 존재를 확인한다.
  최신 절 하나는 면제하므로 한 박자 늦게 잡는다. 태그를 일부러 지워
  그 테스트가 실패하는 것까지 확인했다

버전 사본이 어긋났던 것과 같은 유형이다. 규칙만 두고 확인이 없으면 어긋난다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U227"/>
+  <dimension ref="A1:U228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -18928,6 +18928,114 @@
         </is>
       </c>
     </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>BUG-152</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>릴리즈 태그가 45개 빠져 있었다</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>- rules/release_process.md 가 커밋 뒤에 git tag 와 git push --tags 를 지시하는데 지켜지지 않았다.
+- 릴리즈 노트 절 52개 중 태그가 달린 것은 7개뿐이었다. v1.2.1.0 이후로 45개가 통째로 빠져 있었다.
+- 버전별 코드 상태를 되짚을 수단이 없었다.</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>- 릴리즈마다 태그가 남는다.</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>- 2026-04-08 의 v1.2.1.0 이 마지막 태그였다.</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>1. git tag 목록을 뽑는다.
+2. Release_note.md 의 버전 절 목록과 대조한다.</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>- 태그 7개 대 릴리즈 노트 절 52개. GitHub 릴리즈 페이지도 v1.2.0.0 이 마지막이었다.</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>- 사용자</t>
+        </is>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>원인: - 절차 문서에만 적혀 있고 확인하는 장치가 없었다. 버전 사본이 어긋났던 것과 같은 유형이다.
+수정 내용: - 커밋 메시지의 (vX.X.X.X 표기로 릴리즈 커밋을 찾아 34개를 소급해 달고 푸시했다.
+- 남은 11개(v1.2.2.0 과 v0.x 초기 버전)는 커밋을 특정하지 못해 달지 않았다. 틀린 태그는 없는 태그보다 나쁘다.</t>
+        </is>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>- test_version_consistency.py 에 지난 릴리즈의 태그 존재를 확인하는 테스트를 넣었다. 최신 절 하나는 면제하므로 한 박자 늦게 잡는다.
+- 태그를 일부러 지워 그 테스트가 실패하는 것까지 확인했다.</t>
+        </is>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>- 릴리즈 절차와 태그 이력. 제품 동작은 바뀌지 않는다.</t>
+        </is>
+      </c>
+      <c r="R228" t="inlineStr">
+        <is>
+          <t>System 1.6.7.0</t>
+        </is>
+      </c>
+      <c r="S228" t="inlineStr">
+        <is>
+          <t>System 1.6.7.1</t>
+        </is>
+      </c>
+      <c r="T228" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U228" t="inlineStr">
+        <is>
+          <t>SYM-117</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(report): 리포트 BLOCK 상세, PDF 표 폭, 우선순위별 요약 (v1.6.8.0, SYM-118~122)
- 상세 목록에 FAIL 과 BLOCK 을 함께 싣고 우선순위 높은 순으로 세운다
- PDF 표 폭을 본문 폭에서 계산, 굵은체와 날짜와 N/A 표기 수정
- PDF 폰트로 Pretendard(OFL-1.1)를 backend/fonts 에 포함
- 우선순위별 요약, 분류별 PASS Rate, 직전 수행 대비, 수행자 추가
- 다운로드 파일 이름은 Content-Disposition, 엑셀 PASS Rate 는 숫자 셀
- 이슈 키를 Jira Base URL 로 링크

QA 2인 통과. 미해결: SYM-123 수행 그리드의 이슈 키 링크

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U228"/>
+  <dimension ref="A1:U234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -19036,6 +19036,600 @@
         </is>
       </c>
     </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>BUG-153</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>리포트에 BLOCK 결과의 상세가 빠진다</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>- BLOCK 건수는 요약 카드와 분류 표에 나오지만 어떤 TC 가 왜 막혔는지는 웹 리포트, PDF, 연관 이슈 목록 어디에도 없다
+- BLOCK 만 있는 수행은 '실패 항목이 없습니다' 로 나온다</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>- BLOCK 결과도 TC, 실제 결과, 이슈 링크와 함께 리포트 상세 목록에 실린다</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>- project 116 run 25(BLOCK 2건, 실제 결과 기재): /reports 응답의 top_failures 와 jira_issues 가 빈 배열</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>1. BLOCK 결과가 있고 FAIL 이 없는 수행을 고른다
+2. 리포트 탭에서 그 수행을 선택한다
+3. 주요 실패 항목과 PDF 를 본다</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>- run 25 리포트 JSON: summary.block=2, top_failures=[]</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>- 실서버 팩트체크(QA 2인)</t>
+        </is>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>원인: - routes/reports.py 의 _failed_items 가 result == FAIL 만 조회했다. 엑셀 Results 시트만 전 결과를 실어 BLOCK 상세가 거기에만 있었다
+수정 내용: - FAIL 과 BLOCK 을 함께 조회해 우선순위 높은 순으로 싣고 result 에 실제 값을 넣는다. 연관 이슈도 두 결과에서 모은다(순서 보존, 중복 제거)</t>
+        </is>
+      </c>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_report_content.py 에 BLOCK 만 있는 수행 테스트. ReportView.test.tsx 에 BLOCK 행 표시 테스트</t>
+        </is>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>- 웹 리포트, PDF 리포트, 연관 이슈 목록</t>
+        </is>
+      </c>
+      <c r="R229" t="inlineStr">
+        <is>
+          <t>BE 1.6.4.0</t>
+        </is>
+      </c>
+      <c r="S229" t="inlineStr">
+        <is>
+          <t>System 1.6.8.0 / BE 1.6.5.0 / FE 1.6.5.0</t>
+        </is>
+      </c>
+      <c r="T229" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U229" t="inlineStr">
+        <is>
+          <t>SYM-118</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>BUG-154</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>PDF 리포트 요약 표의 합격률 칸이 페이지 밖으로 잘린다</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>- PDF Summary 표의 Pass Rate 머리글이 'Pas', 값이 '9' 로 잘려 합격률을 읽을 수 없다</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>- 표가 본문 폭 안에 들어오고 합격률이 온전히 보인다</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>- 칸 27mm x 8 = 216mm 로 A4 본문 190mm 를 넘는다. 값이 x=590pt(페이지 폭 595pt)에서 시작한다</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>1. 아무 수행의 PDF 리포트를 받는다
+2. Summary 표 오른쪽 끝을 본다</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>- report_25.pdf 렌더 이미지, pypdf 좌표 x=590.2pt</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>- 실서버 팩트체크(QA 2인)</t>
+        </is>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>원인: - 칸 폭을 숫자로 박아 두고 칸을 늘리면서 합이 본문 폭을 넘었다
+수정 내용: - 칸 폭을 pdf.epw 에서 나눈다. 페이지를 넘는 표는 머리행을 다시 그린다. 굵은체 파일 등록, Version None -&gt; N/A, 날짜 표기, 말줄임 표시도 함께 고쳤다</t>
+        </is>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>- 합격률 값의 x 좌표가 여백선 안인지 보는 테스트. 옛 배치(27mm 고정)로 실패하는 것 확인</t>
+        </is>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>- PDF 리포트</t>
+        </is>
+      </c>
+      <c r="R230" t="inlineStr">
+        <is>
+          <t>BE 1.6.4.0</t>
+        </is>
+      </c>
+      <c r="S230" t="inlineStr">
+        <is>
+          <t>System 1.6.8.0 / BE 1.6.5.0 / FE 1.6.5.0</t>
+        </is>
+      </c>
+      <c r="T230" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U230" t="inlineStr">
+        <is>
+          <t>SYM-119</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>BUG-155</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>한글 폰트가 없는 서버에서 PDF 리포트가 500 오류를 낸다</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>- 한글 폰트가 설치되지 않은 리눅스 서버와 CI 에서 PDF 리포트가 실패한다</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>- 서버 환경과 무관하게 한글이 든 PDF 가 만들어진다</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>- 폰트 탐색이 실패하면 Helvetica 로 떨어지고, 프로젝트명이나 수행명에 한글이 한 글자만 있어도 FPDFUnicodeEncodingException 이 난다</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>- 서버에 맑은 고딕과 나눔고딕이 없다</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>1. 한글 폰트가 없는 환경에서 백엔드를 띄운다
+2. 이름에 한글이 있는 수행의 PDF 리포트를 받는다</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>- FPDF Helvetica 에 한글 cell 출력 시 FPDFUnicodeEncodingException 재현</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(QA1 지적 후 재현)</t>
+        </is>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>원인: - 폰트를 시스템 경로에서만 찾았다. 맑은 고딕은 재배포가 안 돼 레포에 넣을 수 없었다
+수정 내용: - Pretendard(OFL-1.1) Regular/Bold TTF 와 OFL.txt 를 backend/fonts 에 넣고 첫 후보로 쓴다</t>
+        </is>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>- 한글 폰트가 없으면 skip 하던 PDF 테스트를 없애고, 레포 폰트가 실제로 잡히는지 단언한다. CI 에서도 PDF 테스트가 돈다</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>- PDF 리포트(리눅스 배포, CI)</t>
+        </is>
+      </c>
+      <c r="R231" t="inlineStr">
+        <is>
+          <t>BE 1.6.4.0</t>
+        </is>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>System 1.6.8.0 / BE 1.6.5.0 / FE 1.6.5.0</t>
+        </is>
+      </c>
+      <c r="T231" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U231" t="inlineStr">
+        <is>
+          <t>SYM-120</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>BUG-156</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>리포트 다운로드 파일 이름과 날짜, 이슈 링크 표기가 틀리다</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>- 다운로드 파일이 report_번호.pdf 로 저장된다
+- 수행일 칸에 생성일이 나온다
+- 이슈 키만 적은 링크가 href=# 로 걸린다
+- 엑셀 합격률이 문자열이다</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>- 파일 이름이 프로젝트명_Report_R라운드 이고, 생성일과 완료일이 따로 나오고, 이슈 키는 Jira Base URL 로 이어지고, 엑셀 합격률은 숫자다</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>- 브라우저 suggestedFilename 이 report_25.pdf. 엑셀 Summary I7 셀이 문자열 '92.0%'</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>1. 리포트 탭에서 PDF/Excel 을 받는다
+2. 파일 이름과 엑셀 합격률 셀을 본다</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>- Playwright 다운로드 이벤트 suggestedFilename, openpyxl 셀 타입 str</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>- 실서버 팩트체크(QA 2인)</t>
+        </is>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>원인: - 화면이 파일 이름을 직접 정했고, 엑셀에 f-string 으로 넣었고, 링크는 http 가 아니면 # 로 걸었다
+수정 내용: - Content-Disposition 을 읽어 파일 이름을 쓴다(CORS expose_headers 추가). 합격률을 숫자 + 0.0% 서식으로. resolveIssueUrl 로 이슈 키를 링크하고 못 만들면 글자로만 둔다</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>- 파일 이름, 날짜, 링크, 엑셀 숫자 셀 테스트 추가</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>- 리포트 화면, PDF/엑셀 다운로드</t>
+        </is>
+      </c>
+      <c r="R232" t="inlineStr">
+        <is>
+          <t>FE 1.6.4.0</t>
+        </is>
+      </c>
+      <c r="S232" t="inlineStr">
+        <is>
+          <t>System 1.6.8.0 / BE 1.6.5.0 / FE 1.6.5.0</t>
+        </is>
+      </c>
+      <c r="T232" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U232" t="inlineStr">
+        <is>
+          <t>SYM-121</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>ENH-056</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>리포트에 우선순위별 요약과 직전 수행 대비를 싣는다</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>- 리포트는 전체 요약과 분류별 건수만 싣는다. 우선순위별 결과와 직전 수행 대비 변화는 대시보드와 비교 화면에서 따로 봐야 한다</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>- 웹/PDF/엑셀 리포트에 우선순위별 요약, 분류별 PASS Rate, 직전 수행 대비 퇴보/개선, 수행자가 실린다</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>- [ ] 우선순위 높은 것부터 요약되고 빈 우선순위는 한 줄로 모인다
+- [ ] 퇴보/개선 판정이 비교 화면과 같다
+- [ ] 엑셀 Summary 에 같은 표가 있다</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>- 리포트는 밖으로 나가는 산출물이라 받는 사람이 다른 화면을 볼 수 없다. 출시 판단에 필요한 높은 우선순위 실패 수가 리포트에 없다</t>
+        </is>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>- 완료 조건 전부 충족. 변경 건수는 두 런 모두 수행한 TC 만 센다(직전 런이 진행 중이면 NS -&gt; PASS 잡음이 생겨서). 매뉴얼에 차이를 적었다</t>
+        </is>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t>- 출시 판정(Go/No-Go) 기준. 기준을 정해야 해서 뺀다</t>
+        </is>
+      </c>
+      <c r="R233" t="inlineStr">
+        <is>
+          <t>BE 1.6.4.0</t>
+        </is>
+      </c>
+      <c r="S233" t="inlineStr">
+        <is>
+          <t>System 1.6.8.0 / BE 1.6.5.0 / FE 1.6.5.0</t>
+        </is>
+      </c>
+      <c r="T233" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U233" t="inlineStr">
+        <is>
+          <t>SYM-122</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>BUG-157</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>테스트 수행 그리드의 이슈 키가 Jira 링크로 이어지지 않는다</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>- 매뉴얼은 이슈 키를 적으면 Jira Base URL 로 이동한다고 안내하지만 테스트 수행 그리드의 Issue Link 칸은 글자일 뿐이다</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>- 이슈 키 또는 http(s) 주소가 링크로 열린다</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>- TestCaseGrid 는 jiraBaseUrl 을 context 에 넣기만 하고 읽는 렌더러가 없다. TestRunManager 의 issue_link 칸에는 렌더러가 없다</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>1. 프로젝트 설정에 Jira Base URL 을 넣는다
+2. 테스트 수행에서 Issue Link 칸에 PROJ-1 을 적는다
+3. 그 칸을 누른다</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>- grep: jiraBaseUrl 소비 코드 0건. manual.json tcManage.field_issueLink, settings.pi_li2</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>- QA2 팩트체크</t>
+        </is>
+      </c>
+      <c r="R234" t="inlineStr">
+        <is>
+          <t>FE 1.6.5.0</t>
+        </is>
+      </c>
+      <c r="T234" t="inlineStr">
+        <is>
+          <t>미해결</t>
+        </is>
+      </c>
+      <c r="U234" t="inlineStr">
+        <is>
+          <t>SYM-123</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(run): 테스트 수행 시트 이슈 링크 열기 (v1.6.10.0, SYM-123)
- Issue Link 칸에 이슈 키나 주소가 있으면 옆의 ↗ 로 이슈 관리 도구의 이슈를 연다
- ↗ 는 포커스를 받지 않고, 더블클릭과 Enter 가 셀 편집으로 번지지 않게 브라우저 리스너로 막는다
- E2E TC-RUN-023 추가, 매뉴얼과 docs 문구 정리

QA 2인 통과

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -19614,14 +19614,35 @@
           <t>- QA2 팩트체크</t>
         </is>
       </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>- 원인: 테스트 수행 그리드의 issue_link 칸에 렌더러가 없었고, TestCaseGrid 는 jiraBaseUrl 을 context 에 넣기만 하고 읽지 않았다. 매뉴얼만 기능을 약속했다
+- 수정: IssueLinkCell 렌더러가 이슈 키나 주소 옆에 ↗ 를 붙인다(resolveIssueUrl, 리포트와 같은 규칙). ↗ 는 포커스를 받지 않고, 더블클릭과 Enter 가 셀 편집으로 번지지 않게 브라우저 리스너로 막는다</t>
+        </is>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>- IssueLinkCell 단위 테스트 13건(브라우저 리스너 기준 전파, 포커스, 값 변경 뒤 리스너), GridEditorContract 에 렌더러와 trackerUrl 값 계약, E2E TC-RUN-023(↗ 더블클릭, 가운데 클릭 뒤 Enter, 링크 포커스 Enter). 각 테스트는 수정을 빼면 실패하는 것 확인</t>
+        </is>
+      </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>- 테스트 수행 그리드 Issue Link 칸. 매뉴얼과 docs 의 이슈 링크 설명</t>
+        </is>
+      </c>
       <c r="R234" t="inlineStr">
         <is>
           <t>FE 1.6.5.0</t>
         </is>
       </c>
+      <c r="S234" t="inlineStr">
+        <is>
+          <t>System 1.6.10.0 / FE 1.6.7.0</t>
+        </is>
+      </c>
       <c r="T234" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U234" t="inlineStr">

</xml_diff>

<commit_message>
chore(data): 우선순위 옛 값 '중간' 을 '보통' 으로 일괄 변경 (v1.6.10.2, SYM-128)
- ymseo_test TC 98건, 일괄 변경 API 로 변경 이력 98건 기록
- 코드 변경 없음. 변경 전 DB 백업 보관

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U238"/>
+  <dimension ref="A1:U239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -20032,6 +20032,90 @@
         </is>
       </c>
     </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>ENH-059</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>우선순위 옛 값 '중간' 을 '보통' 으로 일괄 변경한다</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>- ymseo_test 프로젝트 TC 98건의 우선순위가 4단계 목록에 없는 옛 값 '중간' 이라 TC 관리와 테스트 수행 그리드에서 색이 입혀지지 않는다</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>- 98건 모두 '보통' 이다. 4단계 목록 밖의 값이 없어진다</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>- [ ] priority='중간' 인 TC 가 0건이다
+- [ ] 바뀐 98건 모두 변경 이력이 남는다
+- [ ] 변경 전 DB 백업이 있다</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>- v1.6.9.0 에서 우선순위를 4단계로 정하면서 '중간' 이 목록 밖 값이 됐다. 사용자 지시</t>
+        </is>
+      </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>- 일괄 변경 API(PUT /testcases/bulk)로 98건 변경. 중간 98-&gt;0, 보통(p23) 0-&gt;98, 변경 이력 6091-&gt;6189(+98, 모두 priority 중간-&gt;보통). 백업 backend/tc_manager.db.bak_20260923_194029_priority</t>
+        </is>
+      </c>
+      <c r="P239" t="inlineStr">
+        <is>
+          <t>- 다른 목록 밖 값(High, Medium, 중요, 핵심 등)과 빈 우선순위 정리</t>
+        </is>
+      </c>
+      <c r="R239" t="inlineStr">
+        <is>
+          <t>System 1.6.10.1</t>
+        </is>
+      </c>
+      <c r="S239" t="inlineStr">
+        <is>
+          <t>System 1.6.10.2(데이터 정리, 코드 변경 없음)</t>
+        </is>
+      </c>
+      <c r="T239" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U239" t="inlineStr">
+        <is>
+          <t>SYM-128</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(ui): 우선순위 글자색 대비, 리포트 빈 값 표기 통일 (v1.6.10.5, SYM-129/130)
- 우선순위 색을 --priority-* 테마 토큰으로 옮겨 그리드 hover/선택까지 AA 4.5:1
- 리포트의 빈 분류/우선순위를 화면 (미분류)/(미지정), 파일 (none), JSON null 로 통일

QA 2인 통과

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U239"/>
+  <dimension ref="A1:U241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -20116,6 +20116,214 @@
         </is>
       </c>
     </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>BUG-160</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>우선순위 글자색이 접근성 대비 기준(4.5:1)에 못 미친다</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>- TC 관리와 테스트 수행 그리드의 우선순위 글자색 일부가 배경과 대비가 낮다</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>- 12px 굵은 글씨라 라이트/다크 테마 모두 카드 배경, 행 hover, 선택 행에서 4.5:1 이상</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>- 고정색이라 다크 '보통' #2563EB 가 카드 위 3.22:1, 다크 '매우 높음' 3.44:1, 라이트 '낮음' 3.3:1</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>1. 다크 테마로 TC 관리를 연다
+2. 우선순위 칸 글자색과 배경색의 대비를 잰다</t>
+        </is>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>- QA2 측정(getComputedStyle, 픽셀 대비), cssTokens 대비 계산</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>- QA2 리뷰</t>
+        </is>
+      </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>원인: - 우선순위 색이 테마와 무관한 고정 hex 였다
+수정 내용: - --priority-* CSS 변수로 옮기고 라이트 #B91C1C/#B54200/#1D4ED8/#166534, 다크 #F87C7C/#FB923C/#60A5FA/#4ADE80. 라이트 '높음' 은 빨강과 구분되는 가장 밝은 주황</t>
+        </is>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>- cssTokens.test.ts 가 테마별 그리드 블록의 hover/선택 값으로 합성한 배경까지 4.5:1 을 검사. priority.test.ts 가 CSS 변수 사용을 고정. 옛 색으로 되돌리면 실패 확인</t>
+        </is>
+      </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>- TC 관리, 테스트 수행 그리드의 우선순위 칸</t>
+        </is>
+      </c>
+      <c r="R240" t="inlineStr">
+        <is>
+          <t>FE 1.6.7.1</t>
+        </is>
+      </c>
+      <c r="S240" t="inlineStr">
+        <is>
+          <t>System 1.6.10.5 / FE 1.6.7.2 / BE 1.6.5.1</t>
+        </is>
+      </c>
+      <c r="T240" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U240" t="inlineStr">
+        <is>
+          <t>SYM-129</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>BUG-161</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>trivial</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>리포트에서 분류와 우선순위가 비어 있는 TC 의 표기가 곳마다 다르다</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>- 분류 없는 TC 가 요약 표는 'Uncategorized', 실패·차단 목록은 '-'. 우선순위도 요약 표 '(미지정)', 목록 '-', 영어 화면에서 목록만 번역 안 됨</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>- 화면은 '(미분류)'/'(미지정)', PDF/엑셀은 '(none)' 로 통일되고 영어 화면은 번역된다</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>- 같은 TC 가 표마다 다른 이름으로 보인다</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>1. 분류나 우선순위가 빈 TC 가 FAIL 인 런의 리포트를 연다
+2. 요약 표와 실패·차단 목록의 표기를 비교한다</t>
+        </is>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>- QA2 리뷰: 요약 표 'Uncategorized' 대 목록 '-', EN 화면 목록 우선순위 '높음'</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>- QA2 리뷰</t>
+        </is>
+      </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>원인: - 백엔드가 분류 요약에서만 이름('Uncategorized')을 정했고, 화면 목록은 따로 '-' 로 대체했다
+수정 내용: - JSON 은 빈 값을 null 로 정규화(요약, 목록 모두). 화면은 i18n 으로 '(미분류)'/'(미지정)' 과 우선순위 번역, PDF/엑셀은 '(none)'</t>
+        </is>
+      </c>
+      <c r="P241" t="inlineStr">
+        <is>
+          <t>- ReportView 테스트(분류/우선순위 표기, 영어 번역), 백엔드 테스트(JSON null, 엑셀·PDF '(none)'). 수정을 빼면 실패 확인</t>
+        </is>
+      </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>- 리포트 화면, PDF, 엑셀 Summary</t>
+        </is>
+      </c>
+      <c r="R241" t="inlineStr">
+        <is>
+          <t>BE 1.6.5.0</t>
+        </is>
+      </c>
+      <c r="S241" t="inlineStr">
+        <is>
+          <t>System 1.6.10.5 / FE 1.6.7.2 / BE 1.6.5.1</t>
+        </is>
+      </c>
+      <c r="T241" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U241" t="inlineStr">
+        <is>
+          <t>SYM-130</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: System 2.0.0.0 릴리즈 노트와 이슈 로그 (PostgreSQL 단일화)
- 버전: System 2.0.0.0, Backend 2.0.0.0, Database 1.0.0.0, Frontend 1.11.0.0
- 이슈 로그에 SYM-136~145 (전환 중 재현·수정한 결함 10건)

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U245"/>
+  <dimension ref="A1:U255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -20744,6 +20744,1040 @@
         </is>
       </c>
     </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>SEC-021</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>동시에 가입하면 첫 관리자가 여러 명 생긴다</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>- 사용자가 없는 DB 에 가입 요청을 동시에 보내면 관리자 계정이 2명 이상 생긴다</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>- 첫 가입자 한 명만 관리자, 나머지는 일반 사용자</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>- 동시 가입 8건 중 관리자 2~5명</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>1. 빈 DB 로 서버를 띄운다
+2. 서로 다른 아이디로 가입 요청 8개를 동시에 보낸다
+3. role=admin 인 사용자 수를 센다</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>- 항상(동시 요청 수 4~8 에서)</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_first_admin_concurrent.py</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(설계 QA 2인) 후 PostgreSQL 에서 동시 요청 테스트로 재현</t>
+        </is>
+      </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>원인: - '사용자 수가 0 이면 관리자' 판정과 INSERT 사이에 잠금이 없다. SQLite 는 쓰기를 직렬화해 드러나지 않았다
+수정 내용: - 판정과 INSERT 를 트랜잭션 범위 advisory lock(FIRST_ADMIN) 안에서 한다. 해시 계산은 잠금 밖</t>
+        </is>
+      </c>
+      <c r="P246" t="inlineStr">
+        <is>
+          <t>- 동시 가입 테스트(잠금을 빼면 실패하는 것 확인)</t>
+        </is>
+      </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>- 새 설치의 첫 가입</t>
+        </is>
+      </c>
+      <c r="R246" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T246" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U246" t="inlineStr">
+        <is>
+          <t>SYM-136</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>SEC-022</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>1회용 코드를 동시 요청으로 여러 번 쓸 수 있다</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>- 계정 찾기·비밀번호 재설정 1회용 코드를 동시에 보내면 여러 요청이 성공한다</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>- 한 요청만 성공, 나머지는 401</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>- 동시 8건 중 4건 성공</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>1. 관리자가 요청을 승인해 코드를 발급한다
+2. 같은 코드로 재설정 요청 8개를 동시에 보낸다</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>- 항상(동시 요청 수 4~8 에서)</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>- test_account_requests 의 동시 사용 테스트 결과 [200]*4</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(설계 QA 2인) 후 PostgreSQL 에서 동시 요청 테스트로 재현</t>
+        </is>
+      </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>원인: - 코드 행을 읽고 사용 처리하는 사이에 행 잠금이 없다
+수정 내용: - 코드 행을 SELECT ... FOR UPDATE 로 읽는다. 승인·거절도 같은 행 잠금</t>
+        </is>
+      </c>
+      <c r="P247" t="inlineStr">
+        <is>
+          <t>- 동시 사용 테스트가 [200]+[401]*7 을 단언</t>
+        </is>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>- 계정 찾기, 비밀번호 재설정</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>SYM-137</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>SEC-023</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>로그인 실패 제한을 동시 요청으로 넘을 수 있다</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>- 실패 횟수 확인과 기록 사이에 다른 요청이 끼어들어 제한보다 많이 시도할 수 있다</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>- 제한 횟수를 넘는 시도는 429</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>- 동시 요청에서 제한을 넘는 시도가 401 로 처리됨</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>1. 같은 아이디로 틀린 비밀번호 로그인을 제한 수보다 많이 동시에 보낸다</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>- 항상(동시 요청 수 4~8 에서)</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_rate_limit.py</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(설계 QA 2인) 후 PostgreSQL 에서 동시 요청 테스트로 재현</t>
+        </is>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>원인: - 실패 기록이 프로세스 메모리에 있어 서버리스 인스턴스끼리 공유되지 않고, 확인과 기록이 원자적이지 않다
+수정 내용: - rate_limit_events 테이블로 옮기고 키 단위 advisory lock 안에서 확인·기록</t>
+        </is>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>- 동시 실패 테스트</t>
+        </is>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>- 로그인, 계정 요청 제출</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T248" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>SYM-138</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>BUG-165</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>같은 수행 결과를 동시에 저장하면 한쪽이 조용히 덮어쓴다</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>- 두 사람이 같은 결과 행을 거의 동시에 저장하면 둘 다 성공하고 먼저 저장한 값이 사라진다</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>- 늦은 저장은 충돌(409)로 알리거나 순서대로 반영</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>- 동시 저장 전부 성공, 마지막 값만 남음</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>1. 같은 수행의 같은 결과 행에 저장 요청 여러 개를 동시에 보낸다</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>- 항상(동시 요청 수 4~8 에서)</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_result_conflict_concurrent.py</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(설계 QA 2인) 후 PostgreSQL 에서 동시 요청 테스트로 재현</t>
+        </is>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>원인: - 기존 행을 읽고 쓰는 사이에 잠금이 없다
+수정 내용: - 수행 단위 advisory lock(RUN_RESULTS) + 기존 행 FOR UPDATE. 결과 가져오기와 동기화도 같은 잠금</t>
+        </is>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t>- 동시 저장 테스트, 잠금 범위 테스트(test_run_results_lock)</t>
+        </is>
+      </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>- 테스트 수행 결과 저장, 결과 가져오기</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U249" t="inlineStr">
+        <is>
+          <t>SYM-139</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>BUG-166</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>동시에 TC 를 복제하면 일부가 409 로 실패한다</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>- 같은 프로젝트에서 TC 복제나 시트 이동이 동시에 들어오면 일부 요청이 409</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>- 모두 성공하고 TC 번호가 겹치지 않는다</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>- 동시 복제 8건 중 일부 409</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>1. TC 가 있는 프로젝트에서 복제 요청 8개를 동시에 보낸다</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>- 항상(동시 요청 수 4~8 에서)</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>- test_tc_clone_concurrent.py</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(설계 QA 2인) 후 PostgreSQL 에서 동시 요청 테스트로 재현</t>
+        </is>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>원인: - 번호 다시 매기기가 프로젝트 단위로 직렬화되지 않는다
+수정 내용: - 구조를 바꾸는 라우트에 프로젝트 쓰기 잠금. 대기 상한(LOCK_WAIT_TIMEOUT_MS)을 넘으면 409 와 안내 문구</t>
+        </is>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t>- 동시 복제 테스트(배리어로 동시 출발), 잠금 범위 테스트</t>
+        </is>
+      </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>- TC 생성·복제·삭제·정렬, 시트 생성·이동·삭제</t>
+        </is>
+      </c>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>SYM-140</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>BUG-167</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>db</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>TC 번호 다시 매기기가 SQLite 전용 임시 테이블에 의존한다</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>- PostgreSQL 에서 번호 다시 매기기가 임시 테이블 문법 차이로 실패하거나 트랜잭션 풀러에서 세션 상태가 깨진다</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>- 두 DB 모두에서 같은 결과</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>- PostgreSQL 전환 시 동작하지 않는 경로</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>1. PostgreSQL 에서 시트의 TC 순서를 바꾼다</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>- 항상(동시 요청 수 4~8 에서)</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>- services/tc_numbering.py 의 옛 구현</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(설계 QA 2인) 후 PostgreSQL 에서 동시 요청 테스트로 재현</t>
+        </is>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>원인: - 고유 제약을 피하려고 임시 테이블에 번호를 계산해 두었다
+수정 내용: - UPDATE 두 번(음수로 비켜 두기 -&gt; 최종 번호)으로 바꿔 세션 상태 없이 처리</t>
+        </is>
+      </c>
+      <c r="P251" t="inlineStr">
+        <is>
+          <t>- 재번호 테스트, SQLite 전용 문법 검사 테스트(test_no_sqlite_in_tests)</t>
+        </is>
+      </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>- TC 정렬, 삭제 후 번호</t>
+        </is>
+      </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>SYM-141</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>BUG-168</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>고급 필터 조건 타입이 다르면 500 이 난다</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>- 숫자 칸(no) 조건에 문자열, in 조건에 목록이 아닌 값을 보내면 500</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>- 400 과 이유</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>- 500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>1. 필터 API 에 {field: no, operator: eq, value: "abc"} 를 보낸다</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>- 항상(동시 요청 수 4~8 에서)</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_filter_types.py</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(설계 QA 2인) 후 PostgreSQL 에서 동시 요청 테스트로 재현</t>
+        </is>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>원인: - SQLite 는 타입이 달라도 비교하지만 PostgreSQL 은 타입 오류를 낸다
+수정 내용: - 숫자 칸은 ASCII 숫자와 정수 범위만 받고, in 은 목록만 받는다. 어기면 400</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>- 타입별 경계 테스트</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>- 고급 필터, 저장된 필터</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>SYM-142</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>BUG-169</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>백엔드 테스트가 개발 DB 를 건드리는지 판정이 SQLite 파일 기준이다</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>- PostgreSQL 로 바꾸면 테스트가 개발 DB 를 쓰는지 판정하지 못해 개발 데이터를 지울 수 있다</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>- 테스트는 세션마다 임시 DB 를 만들고 지운다. 개발 DB 에는 닿지 않는다</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>- 판정이 tc_manager.db 경로 비교라 PostgreSQL 에서는 무력</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>1. DATABASE_URL 을 PostgreSQL 개발 DB 로 두고 백엔드 테스트를 실행한다</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>- 항상(동시 요청 수 4~8 에서)</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>- 옛 conftest.py, dev_db_guard.py</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(설계 QA 2인) 후 PostgreSQL 에서 동시 요청 테스트로 재현</t>
+        </is>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>원인: - 테스트 격리가 SQLite 파일 복사에 기대고 있었다
+수정 내용: - testing_db 가 세션 임시 DB(로컬 호스트만, 쿼리 옵션 거부)를 만들고 지운다. .env 의 DATABASE_URL_DIRECT 재주입도 막음</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>- test_db_isolation, test_testing_db</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>- 백엔드 테스트 전체</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>SYM-143</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>BUG-170</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>API 문서(Swagger) 화면이 빈 화면이다</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>- /docs (이제 /api/docs) 를 열면 아무것도 나오지 않는다</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>- API 목록이 보인다</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>- 빈 화면, 콘솔에 CSP 위반</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>1. 서버를 띄우고 브라우저로 /api/docs 를 연다</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>- 백엔드 CSP script-src 'self' 가 jsdelivr 스크립트와 인라인 초기화 스크립트를 막음</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(QA2)</t>
+        </is>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>원인: - 전역 보안 헤더가 문서 페이지에도 같은 CSP 를 준다
+수정 내용: - /api/docs 에만 CDN 과 인라인 스크립트를 허용하는 CSP. 다른 경로는 그대로</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>- 페이지가 부르는 출처와 CSP 를 대조하는 테스트(test_docs_csp), 브라우저 캡처 확인</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>- API 문서 화면, 관리자 매뉴얼의 Swagger 링크</t>
+        </is>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>SYM-144</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>BUG-171</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>파일을 올린 직후 미리보기가 409 로 실패할 수 있다</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>- 로컬 저장소 구성에서 TC 가져오기 파일을 고르면 가끔 '같은 업로드를 처리하는 중입니다' 로 실패한다</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>- 미리보기가 시트 목록을 보여주고 가져오기가 끝난다</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>- CI E2E 에서 '1개 가져옴' 이 끝내 나오지 않음(재시도 포함 2회 연속)</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>1. 로컬 저장소로 서버를 띄운다
+2. TC 가져오기로 CSV 를 고른다(PUT 직후 미리보기 요청)</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>- 간헐(로컬 8회 0건, CI 2회 연속)</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>- GitHub Actions run 37815839247, 37818104306 의 e2e/uploads.spec.ts:58 실패. 라우트 함수를 직접 불러 반환 시점에 행이 잠겨 있음을 확인(test_upload_hardening)</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>- CI(E2E)</t>
+        </is>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>원인: - 업로드 PUT 이 NOWAIT 행 잠금을 잡고 커밋·롤백 없이 반환한다. FastAPI 는 get_db 정리를 응답 뒤에 해서 잠금이 응답 뒤까지 남는다
+수정 내용: - PUT 이 반환 전에 롤백해 잠금을 푼다. 미리보기와 dry run 도 같은 이유로 반환 전에 롤백</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>- 반환 시점 잠금 해제 테스트 3건, CI 에 E2E 실패 스크린샷 보관 단계</t>
+        </is>
+      </c>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>- 로컬 저장소 구성의 TC 가져오기, 결과 가져오기 미리보기</t>
+        </is>
+      </c>
+      <c r="R255" t="inlineStr">
+        <is>
+          <t>BE 1.10.3.0 (PostgreSQL 전환 브랜치)</t>
+        </is>
+      </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.0 / BE 2.0.0.0 (브랜치 feat/postgresql)</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>SYM-145</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: SYM-6 PostgreSQL 전환 이슈 로그 완료 처리
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -1850,7 +1850,15 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>SQLite 동시성 한계, 프로덕션 환경 대비</t>
+          <t>- SQLite 동시성 한계, 프로덕션 환경 대비
+- 결과: DB 를 PostgreSQL 로 단일화, Vercel + Supabase 배포 구성, SQLite 이관 스크립트(사전 점검·검증·첨부 해시 대조) 추가
+- SQLite 버전은 sqlite-legacy 브랜치(v1.10.3.1)로 동결</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>- 회사 계정 인증(Google 로그인, 가입 승인)은 후속 작업
+- Supabase 컷오버는 인증 작업 뒤</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -1858,9 +1866,14 @@
           <t>0.3.0.0</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>System 2.0.0.0</t>
+        </is>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>미해결</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">

</xml_diff>

<commit_message>
fix: TC 가져오기 E2E 간헐 실패 대응 (SYM-146)
빈 프로젝트 화면이 뜬 뒤에 파일을 고르고, 실패하면 API 오류와 콘솔 오류를
api-and-console-problems.txt 로 남긴다. 원인은 확정하지 못해 다음 실패 때
기록으로 확정한다.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U255"/>
+  <dimension ref="A1:U256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -21791,6 +21791,115 @@
         </is>
       </c>
     </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>BUG-172</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>TC 가져오기 E2E 가 CI 에서 간헐로 실패한다</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>- main 푸시 CI 에서 E2E uploads.spec.ts 의 TC 가져오기 테스트가 재시도까지 실패했다
+- 같은 커밋이 브랜치 CI 와 다음 커밋 CI 에서는 통과했다</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>- 빈 프로젝트에서 CSV 를 고르면 '1개 가져옴' 알림이 뜨고 TC 1건이 생긴다</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>- 15초 동안 알림이 없고 화면은 빈 프로젝트 상태 그대로였다</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>1. main 에 c6e1393 을 푸시해 CI E2E 를 돌린다
+2. uploads.spec.ts 의 TC 가져오기 테스트 결과를 본다</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>- 간헐(CI 4회 중 1회, 로컬 격리 환경 25회 반복 0회)</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>- CI run 37865609420 의 e2e-test-results 아티팩트(빈 프로젝트 화면 캡처)
+- 실패 화면에 API 응답 기록이 없어 어느 요청이 실패했는지 남지 않았다</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>- CI(main 머지 직후 푸시 확인)</t>
+        </is>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>원인: - 확정하지 못했다
+- 후보: 화면 로딩 중에는 툴바의 파일 입력이 있다가 빈 프로젝트 화면의 입력으로 바뀌는데, 테스트가 로딩 완료를 기다리지 않고 파일을 골랐다
+수정 내용: - 빈 프로젝트 화면이 뜬 뒤에 파일을 고른다
+- 실패하면 4xx/5xx API 응답, 실패한 요청, 콘솔 오류를 api-and-console-problems.txt 로 남긴다(CI 아티팩트에 포함)</t>
+        </is>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>- 실패 기록 파일. 재발하면 기록으로 원인을 확정한다
+- 기록 동작은 /api/uploads 에 500 을 주입해 남는 것을 확인했다</t>
+        </is>
+      </c>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>- CI E2E 만. 제품 동작 변경 없음</t>
+        </is>
+      </c>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>System 2.0.0.0</t>
+        </is>
+      </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>- System 2.0.0.1</t>
+        </is>
+      </c>
+      <c r="T256" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U256" t="inlineStr">
+        <is>
+          <t>SYM-146</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: 빈 계정 삭제와 연결된 Google 계정 표시 (SYM-162, SYM-163)
Google 로그인으로 실수로 생긴 빈 계정이 Google 계정과 이메일을 쥐고 있으면
본 계정에 연결해도 빈 계정이 남고, 관리자는 지울 수 없었다.

- 관리자 삭제: 작업 기록(모든 사용자 외래키, API 키 포함)이 없는 계정만.
  계정 잠금과 사용자 행 잠금 안에서 세고 지운다
- Google 연결 때 같은 Google 계정을 쥔 빈 Google 전용 계정은 정리하고 연결
  (account=merged). 이메일이 같다는 이유의 자동 병합은 하지 않는다
- users.google_email(0008): 연결된 Google 주소를 표와 연결 창에 표시
- 비밀번호 초기화 뒤 관리 표 갱신. 렌더마다 새 사용자 객체를 주던 테스트 목이
  이 누락을 가리고 있어 고정 객체로 바꿨다

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U271"/>
+  <dimension ref="A1:U275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -23398,6 +23398,339 @@
         </is>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>ENH-063</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>실수로 생긴 빈 계정을 관리자가 정리할 수 없고 Google 연결 뒤에도 빈 계정이 남는다</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>- Google 로그인을 잘못 눌러 생긴 빈 계정을 지울 방법이 없다. 관리자는 승인 대기 계정만 거절(삭제)할 수 있다
+- 그 빈 계정이 Google 계정을 쥐고 있으면 본 계정에 연결할 수 없고(already_linked), 초기화·중지로 우회해 연결해도 빈 계정이 목록에 남고 이메일을 옮겨 오지 못한다</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>- 관리자 '삭제': 작업 기록이 하나도 없는 계정만 지운다. 본인, 승인 대기, 마지막 관리자는 제외
+- Google 연결 때 같은 Google 계정을 쥔 빈 Google 전용 계정(비밀번호 없음, 기록 없음)은 정리하고 연결한다(account=merged). 현재 계정에 이메일이 없으면 이메일도 옮긴다</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>- [x] DELETE /api/auth/users/{id}, 기록(모든 사용자 외래키, API 키 포함)이 있으면 409
+- [x] 연결 시 빈 Google 전용 계정 정리, 기록·비밀번호·마지막 관리자면 거절
+- [x] 관리 화면 삭제 버튼, 매뉴얼, 체크리스트
+- [x] QA 2인 통과</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>- 시험 배포에서 사용자가 admin 연결을 잊고 Google 로그인해 빈 계정이 생겼고, 화면에서 풀 수 없었다</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>- 삭제와 정리는 계정 잠금과 사용자 행 FOR UPDATE 안에서 기록을 세고 지운다. 배정 저장과 겹치면 삭제가 기다렸다가 409
+- QA 지적으로 비밀번호 초기화 뒤 표 갱신, 테스트 목(렌더마다 새 사용자 객체)이 목록 갱신 누락을 가리던 문제를 함께 고침</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>- 기록이 있는 계정끼리의 병합(기록 이전)
+- 이메일이 같다는 이유의 자동 병합(탈취 방지 원칙 유지)</t>
+        </is>
+      </c>
+      <c r="R272" t="inlineStr">
+        <is>
+          <t>System 2.1.1.0</t>
+        </is>
+      </c>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>- System 2.2.0.0 / BE 2.2.0.0 / FE 1.13.0.0 / DB 1.2.0.0</t>
+        </is>
+      </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>SYM-162</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>ENH-064</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>사용자 관리 표에서 연결된 Google 계정을 확인할 수 없다</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>- 로그인 방식 칸은 '비밀번호 + Google' 만 보여 준다
+- 이메일 칸은 다른 계정이 그 주소를 쥐고 있으면 비어 있어, 어느 Google 계정이 연결됐는지 알 수 없다</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>- users.google_email(0008)에 연결된 Google 주소를 남긴다(가입, 로그인, 연결 때 갱신, 해제·초기화·복구 때 삭제)
+- 표의 로그인 방식 칸과 계정 연결 창에 'Google: 주소' 를 보여 준다. 기능 전에 연결된 계정은 '주소 미기록' 이고 다음 Google 로그인 때 채워진다</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>- [x] 마이그레이션 0008 과 왕복 테스트
+- [x] 표와 연결 창 표시, 화면 캡처 확인
+- [x] QA 2인 통과</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>- 사용자가 admin 에 Google 을 연결했는데 표에서 확인할 수 없다고 지적했다</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>- 시험 배포의 admin 은 다음 Google 로그인 때 주소가 채워진다</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>- 이메일 칸 자체의 의미 변경</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>System 2.1.1.0</t>
+        </is>
+      </c>
+      <c r="S273" t="inlineStr">
+        <is>
+          <t>- System 2.2.0.0 / BE 2.2.0.0 / FE 1.13.0.0 / DB 1.2.0.0</t>
+        </is>
+      </c>
+      <c r="T273" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U273" t="inlineStr">
+        <is>
+          <t>SYM-163</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>BUG-181</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>프로젝트 배정과 계정 삭제가 겹치면 배정 요청이 500 을 낸다</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>- 계정 삭제가 먼저 커밋되면 배정 요청은 존재 확인을 이미 통과해 외래키 오류(IntegrityError)를 처리하지 못한다</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>- 404(사용자를 찾을 수 없음)</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>- 500. 데이터는 손상되지 않는다</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>1. 배정 요청이 사용자 존재 확인을 통과한다
+2. 그 사이 관리자가 그 계정을 삭제하고 커밋한다
+3. 배정 요청이 커밋한다</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>- 미확인(경합)</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>- QA2 코드 검토: routes/members.py 의 멤버 추가와 일괄 배정이 commit 을 IntegrityError 로 감싸지 않는다. 승인 대기 거절(reject_user)도 같은 모양</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>- QA</t>
+        </is>
+      </c>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>BE 2.2.0.0</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t>SYM-164</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>ENH-065</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>프론트 테스트의 로그인 사용자 목이 렌더마다 새 객체를 만들어 목록 갱신 누락을 가린다</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>- accessibility, AccountLinkModal, Header, ProjectListPage, ProjectPage 테스트의 useAuth 목이 호출마다 새 user 객체를 돌려준다
+- [currentUser] 에 걸린 effect 가 렌더마다 다시 돌아, 실제 앱에서는 일어나지 않는 재조회가 테스트에서 일어난다</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>- 목이 실제 AuthContext 처럼 같은 객체를 돌려준다(AdminPage 테스트는 이번에 고침)</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>- [ ] 다섯 파일의 목을 고정 객체로 바꾼다
+- [ ] 바꾼 뒤 드러나는 실패를 결함으로 분류해 고친다</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>- AdminPage 에서 이 목이 '비밀번호 초기화 뒤 목록 갱신 누락' 을 가린 것이 확인됐다</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>- 테스트 도우미 공통화 이상의 구조 변경</t>
+        </is>
+      </c>
+      <c r="R275" t="inlineStr">
+        <is>
+          <t>FE 1.13.0.0</t>
+        </is>
+      </c>
+      <c r="T275" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="U275" t="inlineStr">
+        <is>
+          <t>SYM-165</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Excel 97-2003 파일 가져오기 안내 (SYM-170)
- 내용 첫 8바이트가 OLE2(97-2003 형식, 암호 걸린 .xlsx)면 '.xlsx 로 다시 저장' 안내로 400
- 판정은 이름이 아니라 내용. 이름만 .xls 인 xlsx 는 그대로 읽고, 확장자는 대소문자 무시
- 안내 문구 ko/en 번역
- 이슈 로그: SYM-167~171 기록과 종결
- System 2.2.0.2 / BE 2.2.0.1 / FE 1.13.0.2

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U279"/>
+  <dimension ref="A1:U281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -23898,19 +23898,34 @@
           <t>- 매뉴얼 갱신(System 2.2.0.1) QA 에서 같은 유형의 낡은 수치가 이 파일에 남은 것을 확인. 공개 레포라 외부에서 읽힘</t>
         </is>
       </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>- 초안을 지우지 않고 현재 기준으로 갱신: 계정 발급(Google·이메일·승인), 권한 표, 사용자 관리, PostgreSQL·Alembic, 환경변수, pg_dump 백업, 트러블슈팅(Google, 승인 대기, PDF 폰트), FAQ(포트 8008, 계정 도움 요청, 가져오기 형식·헤더 19행·70여 변형), 변경 이력</t>
+        </is>
+      </c>
       <c r="P277" t="inlineStr">
         <is>
           <t>- 매뉴얼 본문 재구성</t>
         </is>
       </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>- docs/confluence_draft.md</t>
+        </is>
+      </c>
       <c r="R277" t="inlineStr">
         <is>
           <t>System 2.2.0.1 / FE 1.13.0.1</t>
         </is>
       </c>
+      <c r="S277" t="inlineStr">
+        <is>
+          <t>- System 2.2.0.4 / FE 1.13.0.3</t>
+        </is>
+      </c>
       <c r="T277" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U277" t="inlineStr">
@@ -23971,19 +23986,36 @@
           <t>- 매뉴얼 갱신 QA 에서 확인. 운영 매뉴얼 5-3 절의 설명과 그림이 불일치</t>
         </is>
       </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>- 25 번을 '비밀번호 초기화 완료' 창으로 재촬영(capture-auth-manual.spec.ts)
+- 같은 그림을 22 와 같은 화면으로 덮어쓰던 capture-all-manual, capture-readme 의 01/02/22/25 저장 제거
+- md 운영 매뉴얼에 5-5-2 계정 복구 요청 승인 절과 그림 25/39/40 연결</t>
+        </is>
+      </c>
       <c r="P278" t="inlineStr">
         <is>
           <t>- 다른 그림 재촬영</t>
         </is>
       </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>- 운영 매뉴얼 그림 25, 캡처 스크립트 3개, docs/manual_admin_confluence.md</t>
+        </is>
+      </c>
       <c r="R278" t="inlineStr">
         <is>
           <t>System 2.2.0.1 / FE 1.13.0.1</t>
         </is>
       </c>
+      <c r="S278" t="inlineStr">
+        <is>
+          <t>- System 2.2.0.4 / FE 1.13.0.3</t>
+        </is>
+      </c>
       <c r="T278" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U278" t="inlineStr">
@@ -24061,19 +24093,252 @@
           <t>- CI(매뉴얼 갱신 브랜치)</t>
         </is>
       </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>- 원인: 앱의 401 인터셉터(src/api/client.ts)가 window.location 으로 /login 을 연다. reload/goto 의 기본 대기(load)는 외부 폰트까지 기다려서, 401 이 load 보다 먼저 오면 그 이동이 대기 중인 탐색을 끊는다
+- 수정: e2e/nav.ts 도우미가 응답 도착(commit)까지만 기다리고 ERR_ABORTED 만 삼킨다. 사용 중지 테스트, 미로그인 리다이렉트 테스트 2곳(auth, regression-full)에 적용. 사용 중지 테스트에 재로그인 시 '사용이 중지된 계정입니다.' 단언 추가</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>- 같은 패턴을 도우미 하나로 모음. 로컬 격리 환경에서 세 테스트 5회 반복 15/15 통과
+- 결정적 재현은 못 함(폰트 지연 주입으로 옛 코드 실패 2회 관측)</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>- E2E 3개 테스트</t>
+        </is>
+      </c>
       <c r="R279" t="inlineStr">
         <is>
           <t>System 2.2.0.1</t>
         </is>
       </c>
+      <c r="S279" t="inlineStr">
+        <is>
+          <t>- System 2.2.0.3</t>
+        </is>
+      </c>
       <c r="T279" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U279" t="inlineStr">
         <is>
           <t>SYM-169</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>BUG-184</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Excel 97-2003(.xls) 파일을 가져오면 이유 없이 'Failed to read Excel file' 로 실패한다</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>- TC 가져오기 파일 선택기와 서버가 .xls 를 받지만, 실제 97-2003 형식 파일은 읽지 못하고 일반 오류만 낸다</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>- 읽을 수 없는 형식이면 이유와 해결 방법(.xlsx 로 다시 저장)을 안내한다</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>- 400 'Failed to read Excel file'</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>1. Excel 97-2003 통합 문서(.xls)를 준비한다
+2. TC 관리에서 가져오기로 그 파일을 고른다</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>- services/import_service.py 가 openpyxl.load_workbook 만 쓰고 xlrd 의존이 없다
+- OLE2 서명으로 시작하는 바이트를 load_workbook 에 넣으면 BadZipFile</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>- QA(매뉴얼 후속 수정의 Codex·QA2 지적)</t>
+        </is>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>원인: - openpyxl 은 OOXML(zip)만 읽는다. 97-2003 형식(OLE2/BIFF)과 암호가 걸린 .xlsx(OLE2 EncryptedPackage)는 읽기에서 예외가 나고 일반 문구로 바뀌었다
+수정 내용: - 내용 첫 8바이트가 OLE2 서명이면 안내 문구(XLS_NOT_SUPPORTED)로 400. 판정은 이름이 아니라 내용으로 해서 이름만 .xls 인 xlsx 는 그대로 읽힌다
+- 확장자 판정을 대소문자 무시로 변경(TC.XLSX 허용)
+- 안내 문구 ko/en 번역 추가</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_import_xls.py 5건(옛 형식 거절, 이름만 .xls 인 xlsx 읽기, 이름이 .xlsx 인 OLE2 거절, 대문자 확장자, 그 외 확장자)
+- errorMessage-upload.test.ts 에 문구 번역 확인 추가</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>- TC 가져오기 미리보기와 가져오기(직접 업로드, upload_id 모두)</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>BE 2.2.0.0</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr">
+        <is>
+          <t>- System 2.2.0.2 / BE 2.2.0.1 / FE 1.13.0.2</t>
+        </is>
+      </c>
+      <c r="T280" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U280" t="inlineStr">
+        <is>
+          <t>SYM-170</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>BUG-185</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>trivial</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>etc</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>DB 설정 단위 테스트가 Windows 에서 하위 프로세스 한글 출력이 깨져 실패한다</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_db_config.py 의 원격 직결 주소 거절 테스트가 Windows 로컬에서만 실패한다(CI 리눅스는 통과)</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>- 운영체제와 무관하게 통과한다</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>- 오류 문구의 한글이 U+FFFD 로 깨져 '원격' 포함 단언이 실패</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>1. Windows 에서 PYTHONUTF8 없이 python -m pytest tests_unit/test_db_config.py 를 실행한다</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>- 항상(Windows)</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>- PYTHONUTF8=1 이면 6건 통과, 없으면 1건 실패</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>- 로컬 전체 테스트 실행</t>
+        </is>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>원인: - 부모는 UTF-8 로 디코딩하는데 자식 파이썬은 Windows 기본 코드페이지(cp949)로 stderr 를 쓴다
+수정 내용: - 두 하위 프로세스 환경에 PYTHONIOENCODING=utf-8</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>- 없음(테스트 자체의 수정). 다른 하위 프로세스 테스트는 같은 패턴이 없음을 확인</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>- 로컬 테스트만</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>System 2.2.0.1</t>
+        </is>
+      </c>
+      <c r="S281" t="inlineStr">
+        <is>
+          <t>- System 2.2.0.3</t>
+        </is>
+      </c>
+      <c r="T281" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U281" t="inlineStr">
+        <is>
+          <t>SYM-171</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: 관리자 API 키 계정 관리 차단과 입력 오류 응답 수정 (SYM-172, SYM-173, SYM-164, SYM-161)
- 계정 관리 8개 API 를 관리자 로그인 세션 전용으로
- 72바이트 넘는 비밀번호와 잘못된 대시보드 날짜가 500 대신 401/400
- 배정 커밋 경합 404/400, 업로드 PUT 배포 모드 판정과 잠금 해제

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U281"/>
+  <dimension ref="A1:U283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -23377,19 +23377,35 @@
           <t>- 배포 환경에서 잘못 불린 요청이 잠금을 쥔 채 외부 호출을 기다린다</t>
         </is>
       </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>* 저장소에 direct_upload 속성(Local False, Supabase True)을 두고 PUT 라우트가 행 잠금 전에 이 값으로 판정해 400 을 낸다. 서명 주소 발급 호출이 없어졌다
+* 409(이미 올림)와 413(상한 초과) 응답 전에도 롤백해 행 잠금을 바로 푼다</t>
+        </is>
+      </c>
       <c r="P271" t="inlineStr">
         <is>
           <t>- 업로드 흐름 재설계</t>
         </is>
       </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>* 로컬 저장소 업로드 PUT 라우트. 테스트 tests_unit/test_upload_put_direct_mode.py</t>
+        </is>
+      </c>
       <c r="R271" t="inlineStr">
         <is>
           <t>BE 2.1.1.0</t>
         </is>
       </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>* BE 2.2.1.0</t>
+        </is>
+      </c>
       <c r="T271" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U271" t="inlineStr">
@@ -23641,14 +23657,35 @@
           <t>- QA</t>
         </is>
       </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>원인: * 존재 확인과 커밋 사이에 계정이 지워지면 외래키 오류가 난다. 실제 응답은 500 이 아니라 전역 IntegrityError 핸들러의 409 '데이터 제약 조건에 걸렸습니다' 였다(재현 테스트로 확인)
+수정 내용: * routes/members.py \_commit_assignment: 커밋 실패 시 롤백 후 계정이 없으면 404, 프로젝트가 없으면 404, 이미 멤버면 400, 그 밖은 409 '다른 요청과 겹쳤습니다'. 멤버 추가와 전체 배정에 적용</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>* tests_unit/test_member_assign_race.py: 커밋 직전 다른 연결로 계정을 지우는 경합 2건, 같은 사용자 동시 추가 1건(수정 전 코드에서 3건 실패)</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>* 프로젝트 멤버 추가, 전체 프로젝트 일괄 배정</t>
+        </is>
+      </c>
       <c r="R274" t="inlineStr">
         <is>
           <t>BE 2.2.0.0</t>
         </is>
       </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>* BE 2.2.1.0</t>
+        </is>
+      </c>
       <c r="T274" t="inlineStr">
         <is>
-          <t>진행중</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="U274" t="inlineStr">
@@ -24339,6 +24376,216 @@
       <c r="U281" t="inlineStr">
         <is>
           <t>SYM-171</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>SEC-029</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>관리자 API 키로 계정 승인과 역할 변경을 할 수 있다</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>- 계정 관리 라우트 7개(approve, reject, disable, enable, release-email, delete, role)와 복구 요청 거절이 role_required("admin") 만 보고 세션 전용 검사가 없다</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>- API 키로 부르면 403. 계정 관리는 관리자 로그인 세션으로만 한다</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>- 관리자 키로 대기 계정을 승인하고 role 을 admin 으로 올릴 수 있다. 키를 폐기해도 올린 관리자 계정은 남는다</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>1. 관리자 세션으로 API 키를 발급한다
+2. 그 키로 POST /api/auth/users/{id}/approve, PUT /api/auth/users/{id}/role {"role":"admin"} 을 보낸다
+3. 200 이 오고 대상 계정이 관리자가 된다</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_api_keys.py::test_관리자_키로는_계정을_관리하지_못한다 8건이 수정 전 코드에서 전부 실패</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(사내 도입 전 보안 감사)</t>
+        </is>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>원인: - 비밀번호 초기화와 복구 승인만 get_session_user 를 거쳤다. 나머지 계정 관리 라우트는 키 인증을 그대로 받았다
+수정 내용: - auth.admin_session_required(관리자 + 세션 전용) 를 만들어 8개 라우트에 건다</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>- 8개 경로를 키로 호출하면 403 인지 보는 표 테스트</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>- 계정 관리 API. 웹 화면 동작은 그대로</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>BE 2.2.0.1</t>
+        </is>
+      </c>
+      <c r="S282" t="inlineStr">
+        <is>
+          <t>BE 2.2.1.0</t>
+        </is>
+      </c>
+      <c r="T282" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U282" t="inlineStr">
+        <is>
+          <t>SYM-172</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>BUG-186</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>긴 비밀번호와 잘못된 대시보드 날짜가 500 을 낸다</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>- bcrypt 5.0 이 72바이트 초과 입력에 ValueError 를 낸다
+- 대시보드 date_from/date_to 파싱 실패가 ValueError 로 남는다</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>- 로그인은 401(실패 횟수 기록), 가입·변경은 400 안내, 날짜는 400</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>- 로그인(ASCII 73자, 한글 25자), 가입, 비밀번호 변경, 코드 초기화, 대시보드 6개 API 가 500</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>1. 로그인에 한글 25자 비밀번호를 넣는다
+2. GET 대시보드 summary 에 date_to=2026-10-01T00:00 을 준다</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>- 항상</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>- tests_unit/test_password_bytes.py, test_dashboard_date_params.py 가 수정 전 코드에서 실패</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>- 코드 리뷰(사내 도입 전 감사)</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>원인: - 비밀번호 바이트 상한과 날짜 형식을 검증하지 않았다
+수정 내용: - verify_password 는 초과를 틀린 비밀번호로(더미 대조로 응답 시간 유지), 새 비밀번호는 ensure_password_fits 로 400. 대시보드 날짜는 400</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>- 경계값(정확히 72바이트) 포함 테스트</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>- 로그인, 가입, 비밀번호 변경, 계정 복구, 대시보드</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>BE 2.2.0.1</t>
+        </is>
+      </c>
+      <c r="S283" t="inlineStr">
+        <is>
+          <t>BE 2.2.1.0</t>
+        </is>
+      </c>
+      <c r="T283" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U283" t="inlineStr">
+        <is>
+          <t>SYM-173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: 이슈 로그에 SYM-198, SYM-199 종결 기록
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Issue_list.xlsx
+++ b/Issue_list.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U306"/>
+  <dimension ref="A1:U309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -26936,6 +26936,273 @@
         </is>
       </c>
     </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>ENH-072</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Claude 스타트업 프로그램 지원용 회사소개 페이지 추가</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>- 제품 소개 자료는 portfolio/YM_TestCase.html, PDF, PPTX 와 README 뿐이다
+- 비로그인 라우트는 /login, /register, /account-help, /reset-password 뿐이고 / 는 /projects 로 보낸다. 외부에 보여줄 회사/제품 소개 페이지가 없다</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>- ym-testcase 에서 회사(팀)와 제품을 소개하는 공개 페이지에 접근할 수 있다
+- Claude 스타트업 프로그램 지원서에 이 페이지 URL 을 적을 수 있다</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>- [ ] 로그인 없이 접근 가능한 회사소개 페이지가 배포 URL 에 있다
+- [ ] 제품 개요, 주요 기능, 스크린샷, 팀/연락처가 들어간다
+- [ ] 프로그램 지원 요건(웹사이트 항목 등)을 확인하고 그에 맞춘다
+- [ ] 페이지 문구가 deslop 검사를 통과한다
+- [ ] QA 2인 검증과 스크린샷 확인을 마친다</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>- 지금 착수하지 않는다. Claude 스타트업 프로그램 지원 시점에 착수한다(백로그)
+- 지원서에 회사/제품 웹사이트를 요구할 때 보여줄 페이지가 없다</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>- 지원서 작성과 제출 자체
+- 기존 앱 화면 레이아웃 변경</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>System 2.2.5.1</t>
+        </is>
+      </c>
+      <c r="T307" t="inlineStr">
+        <is>
+          <t>진행중</t>
+        </is>
+      </c>
+      <c r="U307" t="inlineStr">
+        <is>
+          <t>SYM-197</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>SEC-032</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>security</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>일반 사용자가 프로젝트를 만들 수 없다</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>- 프로젝트 생성 API 가 시스템 역할 qa_manager 이상만 허용한다(POST /api/projects 403)
+- 프로젝트 목록 화면의 '+ 새 프로젝트' 버튼이 qa_manager 이상에게만 보인다</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>- 로그인한 사용자는 누구나 프로젝트를 만든다
+- 만든 사람은 그 프로젝트의 admin 멤버로 등록된다(기존 규칙 유지)
+- 프로젝트 일괄 삭제 체크박스는 지금처럼 qa_manager 이상에게만 보인다</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>- [ ] role=user 계정의 POST /api/projects 가 201 이고 생성자가 admin 멤버로 들어간다
+- [ ] 일반 사용자 화면에 '+ 새 프로젝트' 버튼이 보이고 일괄 삭제 체크박스는 안 보인다
+- [ ] 매뉴얼의 '생성은 Admin 만' 문구와 권한 표가 바뀐 규칙과 맞다</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>- 사용자 요청. 팀원이 자기 업무용 프로젝트를 만들 때마다 관리자에게 부탁해야 한다</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>* `POST /api/projects` 를 로그인 사용자 전체에 허용. 만든 사람은 Project Admin 멤버로 등록
+* 프로젝트 목록의 '+ 새 프로젝트' 버튼을 모든 사용자에게 표시. 일괄 삭제 체크박스는 QA Manager 이상 유지
+* 생성 허용으로 멤버 후보 목록이 사실상 전원에게 열리므로 `available-users` 를 사용 중 계정의 id, 아이디, 표시 이름으로 축소
+* 시스템 관리자가 아니면 사용 중이 아닌 계정의 멤버 추가를 404 로 거절(id 를 넣어 보며 숨긴 계정을 알아내는 경로 차단)
+* 사용자·운영 매뉴얼의 생성 권한 경고문, 권한 표, 역할 요약, API 목록 갱신
+* 완료 조건 3개 충족. 남은 정책 결정: 일반 사용자가 만든 프로젝트의 공개 기본값, 이메일 가입 계정은 아이디가 이메일이라 후보 목록에 보임</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>- 생성 권한을 끄는 환경변수 스위치
+- 사용자별 프로젝트 개수 상한</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>System 2.2.5.1 / BE 2.2.3.0 / FE 1.13.3.0</t>
+        </is>
+      </c>
+      <c r="S308" t="inlineStr">
+        <is>
+          <t>* System 2.2.6.0 / BE 2.2.4.0 / FE 1.13.4.0 (커밋: 533c34c)</t>
+        </is>
+      </c>
+      <c r="T308" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U308" t="inlineStr">
+        <is>
+          <t>SYM-198</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>ENH-073</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>frontend</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>시트를 통째로 복사하는 기능이 없다</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>- 시트는 추가, 이름 변경, 이동, 삭제만 된다
+- 같은 구성의 시트가 필요하면 TC 를 전부 골라 복제한 뒤 시트를 옮기거나 엑셀로 내보내 다시 가져와야 한다</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>- 시트 트리의 시트 행에 복사 버튼이 생긴다
+- 누르면 같은 부모 아래, 원본 바로 다음에 '&lt;원본&gt; (복사)' 시트가 생기고 원본의 살아 있는 TC 가 같은 순서로 들어간다
+- 복사한 TC 는 새 TC ID(&lt;원본 ID&gt;-copy)를 받는다. 수행 결과, 변경 이력, 첨부는 복사하지 않는다</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>- [ ] POST /sheets/{id}/copy 가 새 시트와 TC 를 만들고 번호가 1 부터 이어진다
+- [ ] 이름이 겹치면 (복사 2), (복사 3) 으로 비어 있는 이름을 찾는다. 100자 상한을 넘지 않는다
+- [ ] 폴더는 복사를 거부한다(400). 프로젝트 admin 이 아니면 403
+- [ ] 진행 중인 전체 범위 수행에 복사한 TC 가 NS 로 들어간다
+- [ ] 시트 트리에 복사 버튼이 보이고 누르면 새 시트가 선택된다</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>- 사용자 요청. 회차별·플랫폼별로 같은 TC 묶음을 따로 관리하려는 수요</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>* `POST /api/projects/{id}/testcases/sheets/{sheet_id}/copy` 와 시트 트리 복사 버튼(키보드 Enter/Space 가능) 추가
+* 원본 바로 다음 자리에 `&lt;원본&gt; (복사)`, 겹치면 `(복사 N)`. 시트 행 없이 TC 만 남은 이름도 피함. 100자 상한
+* 살아 있는 TC 를 No 1 부터 복제, TC ID 는 TC 복제와 같은 `-copy` 규칙. 수행 결과, 변경 이력, 첨부는 복사하지 않음
+* 진행 중인 전체 범위 수행 동기화까지 한 트랜잭션. 동기화가 실패하면 복사 전체 취소
+* 완료 조건 5개 충족. '기본' 시트 하나뿐인 프로젝트는 원래 사이드바가 없어 복사 버튼도 보이지 않음(기존 호환 모드, 범위 밖)</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>- 폴더(하위 시트 포함) 복사
+- 다른 프로젝트로 복사</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>System 2.2.5.1 / BE 2.2.3.0 / FE 1.13.3.0</t>
+        </is>
+      </c>
+      <c r="S309" t="inlineStr">
+        <is>
+          <t>* System 2.2.6.0 / BE 2.2.4.0 / FE 1.13.4.0 (커밋: 533c34c)</t>
+        </is>
+      </c>
+      <c r="T309" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="U309" t="inlineStr">
+        <is>
+          <t>SYM-199</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>